<commit_message>
Line 1 and 2 start time data
</commit_message>
<xml_diff>
--- a/data/subway/TTC_start_times.xlsx
+++ b/data/subway/TTC_start_times.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michelle/Documents/GitHub/TardyTerminatorCommittee/data/subway/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{787F5A2D-6AD6-0F43-898E-11E422BDA4BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82D5317F-D68C-7D46-9958-67793484EE47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-15440" yWindow="-28300" windowWidth="30200" windowHeight="28180" xr2:uid="{CE12AB93-EB51-0545-9571-363BDCFCA93A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="84">
   <si>
     <t>Station</t>
   </si>
@@ -688,40 +688,40 @@
         <v>23</v>
       </c>
       <c r="F1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" t="s">
+        <v>52</v>
+      </c>
+      <c r="J1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="M1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="N1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="O1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="P1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="Q1" t="s">
         <v>48</v>
-      </c>
-      <c r="L1" t="s">
-        <v>49</v>
-      </c>
-      <c r="M1" t="s">
-        <v>50</v>
-      </c>
-      <c r="N1" t="s">
-        <v>51</v>
-      </c>
-      <c r="O1" t="s">
-        <v>52</v>
-      </c>
-      <c r="P1" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
@@ -741,40 +741,40 @@
         <v>14</v>
       </c>
       <c r="F2" s="1">
+        <v>0.2298611111111111</v>
+      </c>
+      <c r="G2" s="1">
+        <v>5.5555555555555552E-2</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0.23749999999999999</v>
+      </c>
+      <c r="I2" s="1">
+        <v>5.5555555555555552E-2</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0.32916666666666666</v>
+      </c>
+      <c r="K2" s="1">
+        <v>5.5555555555555552E-2</v>
+      </c>
+      <c r="L2" s="1">
         <v>0.24166666666666667</v>
       </c>
-      <c r="G2" s="1">
+      <c r="M2" s="1">
         <v>9.7916666666666666E-2</v>
       </c>
-      <c r="H2" s="1">
+      <c r="N2" s="1">
         <v>0.25277777777777777</v>
       </c>
-      <c r="I2" s="1">
+      <c r="O2" s="1">
         <v>9.4444444444444442E-2</v>
       </c>
-      <c r="J2" s="1">
+      <c r="P2" s="1">
         <v>0.34722222222222221</v>
       </c>
-      <c r="K2" s="1">
+      <c r="Q2" s="1">
         <v>9.4444444444444442E-2</v>
-      </c>
-      <c r="L2" s="1">
-        <v>0.2298611111111111</v>
-      </c>
-      <c r="M2" s="1">
-        <v>5.5555555555555552E-2</v>
-      </c>
-      <c r="N2" s="1">
-        <v>0.23749999999999999</v>
-      </c>
-      <c r="O2" s="1">
-        <v>5.5555555555555552E-2</v>
-      </c>
-      <c r="P2" s="1">
-        <v>0.32916666666666666</v>
-      </c>
-      <c r="Q2" s="1">
-        <v>5.5555555555555552E-2</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
@@ -794,40 +794,40 @@
         <v>41</v>
       </c>
       <c r="F3" s="1">
+        <v>0.23125000000000001</v>
+      </c>
+      <c r="G3" s="1">
+        <v>5.6944444444444443E-2</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0.2388888888888889</v>
+      </c>
+      <c r="I3" s="1">
+        <v>5.6944444444444443E-2</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0.33055555555555555</v>
+      </c>
+      <c r="K3" s="1">
+        <v>5.6944444444444443E-2</v>
+      </c>
+      <c r="L3" s="1">
         <v>0.23819444444444443</v>
       </c>
-      <c r="G3" s="1">
+      <c r="M3" s="1">
         <v>9.4444444444444442E-2</v>
       </c>
-      <c r="H3" s="1">
+      <c r="N3" s="1">
         <v>0.25069444444444444</v>
       </c>
-      <c r="I3" s="1">
+      <c r="O3" s="1">
         <v>9.2361111111111116E-2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="P3" s="1">
         <v>0.34513888888888888</v>
       </c>
-      <c r="K3" s="1">
+      <c r="Q3" s="1">
         <v>9.2361111111111116E-2</v>
-      </c>
-      <c r="L3" s="1">
-        <v>0.23125000000000001</v>
-      </c>
-      <c r="M3" s="1">
-        <v>5.6944444444444443E-2</v>
-      </c>
-      <c r="N3" s="1">
-        <v>0.2388888888888889</v>
-      </c>
-      <c r="O3" s="1">
-        <v>5.6944444444444443E-2</v>
-      </c>
-      <c r="P3" s="1">
-        <v>0.33055555555555555</v>
-      </c>
-      <c r="Q3" s="1">
-        <v>5.6944444444444443E-2</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
@@ -847,40 +847,40 @@
         <v>14</v>
       </c>
       <c r="F4" s="1">
+        <v>0.2326388888888889</v>
+      </c>
+      <c r="G4" s="1">
+        <v>5.7638888888888892E-2</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0.23958333333333334</v>
+      </c>
+      <c r="I4" s="1">
+        <v>5.7638888888888892E-2</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0.33124999999999999</v>
+      </c>
+      <c r="K4" s="1">
+        <v>5.7638888888888892E-2</v>
+      </c>
+      <c r="L4" s="1">
         <v>0.23749999999999999</v>
       </c>
-      <c r="G4" s="1">
+      <c r="M4" s="1">
         <v>9.375E-2</v>
       </c>
-      <c r="H4" s="1">
+      <c r="N4" s="1">
         <v>0.24930555555555556</v>
       </c>
-      <c r="I4" s="1">
+      <c r="O4" s="1">
         <v>9.0972222222222218E-2</v>
       </c>
-      <c r="J4" s="1">
+      <c r="P4" s="1">
         <v>0.34375</v>
       </c>
-      <c r="K4" s="1">
+      <c r="Q4" s="1">
         <v>9.0972222222222218E-2</v>
-      </c>
-      <c r="L4" s="1">
-        <v>0.2326388888888889</v>
-      </c>
-      <c r="M4" s="1">
-        <v>5.7638888888888892E-2</v>
-      </c>
-      <c r="N4" s="1">
-        <v>0.23958333333333334</v>
-      </c>
-      <c r="O4" s="1">
-        <v>5.7638888888888892E-2</v>
-      </c>
-      <c r="P4" s="1">
-        <v>0.33124999999999999</v>
-      </c>
-      <c r="Q4" s="1">
-        <v>5.7638888888888892E-2</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
@@ -903,37 +903,37 @@
         <v>0.23472222222222222</v>
       </c>
       <c r="G5" s="1">
-        <v>9.0972222222222218E-2</v>
+        <v>5.9722222222222225E-2</v>
       </c>
       <c r="H5" s="1">
-        <v>0.24722222222222223</v>
+        <v>0.24166666666666667</v>
       </c>
       <c r="I5" s="1">
-        <v>8.8888888888888892E-2</v>
+        <v>5.9722222222222225E-2</v>
       </c>
       <c r="J5" s="1">
-        <v>0.34166666666666667</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="K5" s="1">
-        <v>8.8888888888888892E-2</v>
+        <v>5.9722222222222225E-2</v>
       </c>
       <c r="L5" s="1">
         <v>0.23472222222222222</v>
       </c>
       <c r="M5" s="1">
-        <v>5.9722222222222225E-2</v>
+        <v>9.0972222222222218E-2</v>
       </c>
       <c r="N5" s="1">
-        <v>0.24166666666666667</v>
+        <v>0.24722222222222223</v>
       </c>
       <c r="O5" s="1">
-        <v>5.9722222222222225E-2</v>
+        <v>8.8888888888888892E-2</v>
       </c>
       <c r="P5" s="1">
-        <v>0.33333333333333331</v>
+        <v>0.34166666666666667</v>
       </c>
       <c r="Q5" s="1">
-        <v>5.9722222222222225E-2</v>
+        <v>8.8888888888888892E-2</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
@@ -953,40 +953,40 @@
         <v>41</v>
       </c>
       <c r="F6" s="1">
+        <v>0.23680555555555555</v>
+      </c>
+      <c r="G6" s="1">
+        <v>6.1805555555555558E-2</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0.24374999999999999</v>
+      </c>
+      <c r="I6" s="1">
+        <v>6.1805555555555558E-2</v>
+      </c>
+      <c r="J6" s="1">
+        <v>0.33541666666666664</v>
+      </c>
+      <c r="K6" s="1">
+        <v>6.1805555555555558E-2</v>
+      </c>
+      <c r="L6" s="1">
         <v>0.23749999999999999</v>
       </c>
-      <c r="G6" s="1">
+      <c r="M6" s="1">
         <v>8.8888888888888892E-2</v>
       </c>
-      <c r="H6" s="1">
+      <c r="N6" s="1">
         <v>0.24513888888888888</v>
       </c>
-      <c r="I6" s="1">
+      <c r="O6" s="1">
         <v>8.6805555555555552E-2</v>
       </c>
-      <c r="J6" s="1">
+      <c r="P6" s="1">
         <v>0.33958333333333335</v>
       </c>
-      <c r="K6" s="1">
+      <c r="Q6" s="1">
         <v>8.6805555555555552E-2</v>
-      </c>
-      <c r="L6" s="1">
-        <v>0.23680555555555555</v>
-      </c>
-      <c r="M6" s="1">
-        <v>6.1805555555555558E-2</v>
-      </c>
-      <c r="N6" s="1">
-        <v>0.24374999999999999</v>
-      </c>
-      <c r="O6" s="1">
-        <v>6.1805555555555558E-2</v>
-      </c>
-      <c r="P6" s="1">
-        <v>0.33541666666666664</v>
-      </c>
-      <c r="Q6" s="1">
-        <v>6.1805555555555558E-2</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
@@ -1006,40 +1006,40 @@
         <v>41</v>
       </c>
       <c r="F7" s="1">
-        <v>0.23472222222222222</v>
+        <v>0.2388888888888889</v>
       </c>
       <c r="G7" s="1">
-        <v>8.611111111111111E-2</v>
+        <v>6.458333333333334E-2</v>
       </c>
       <c r="H7" s="1">
-        <v>0.24305555555555555</v>
+        <v>0.24583333333333332</v>
       </c>
       <c r="I7" s="1">
-        <v>8.4722222222222227E-2</v>
+        <v>6.3888888888888884E-2</v>
       </c>
       <c r="J7" s="1">
         <v>0.33750000000000002</v>
       </c>
       <c r="K7" s="1">
+        <v>6.3888888888888884E-2</v>
+      </c>
+      <c r="L7" s="1">
+        <v>0.23472222222222222</v>
+      </c>
+      <c r="M7" s="1">
+        <v>8.611111111111111E-2</v>
+      </c>
+      <c r="N7" s="1">
+        <v>0.24305555555555555</v>
+      </c>
+      <c r="O7" s="1">
         <v>8.4722222222222227E-2</v>
-      </c>
-      <c r="L7" s="1">
-        <v>0.2388888888888889</v>
-      </c>
-      <c r="M7" s="1">
-        <v>6.458333333333334E-2</v>
-      </c>
-      <c r="N7" s="1">
-        <v>0.24583333333333332</v>
-      </c>
-      <c r="O7" s="1">
-        <v>6.3888888888888884E-2</v>
       </c>
       <c r="P7" s="1">
         <v>0.33750000000000002</v>
       </c>
       <c r="Q7" s="1">
-        <v>6.3888888888888884E-2</v>
+        <v>8.4722222222222227E-2</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
@@ -1059,40 +1059,40 @@
         <v>41</v>
       </c>
       <c r="F8" s="1">
+        <v>0.24027777777777778</v>
+      </c>
+      <c r="G8" s="1">
+        <v>6.5972222222222224E-2</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0.24652777777777779</v>
+      </c>
+      <c r="I8" s="1">
+        <v>6.458333333333334E-2</v>
+      </c>
+      <c r="J8" s="1">
+        <v>0.33819444444444446</v>
+      </c>
+      <c r="K8" s="1">
+        <v>6.458333333333334E-2</v>
+      </c>
+      <c r="L8" s="1">
         <v>0.25972222222222224</v>
       </c>
-      <c r="G8" s="1">
+      <c r="M8" s="1">
         <v>8.4722222222222227E-2</v>
       </c>
-      <c r="H8" s="1">
+      <c r="N8" s="1">
         <v>0.25694444444444442</v>
       </c>
-      <c r="I8" s="1">
+      <c r="O8" s="1">
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="P8" s="1">
         <v>0.34861111111111109</v>
       </c>
-      <c r="K8" s="1">
+      <c r="Q8" s="1">
         <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="L8" s="1">
-        <v>0.24027777777777778</v>
-      </c>
-      <c r="M8" s="1">
-        <v>6.5972222222222224E-2</v>
-      </c>
-      <c r="N8" s="1">
-        <v>0.24652777777777779</v>
-      </c>
-      <c r="O8" s="1">
-        <v>6.458333333333334E-2</v>
-      </c>
-      <c r="P8" s="1">
-        <v>0.33819444444444446</v>
-      </c>
-      <c r="Q8" s="1">
-        <v>6.458333333333334E-2</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
@@ -1112,40 +1112,40 @@
         <v>41</v>
       </c>
       <c r="F9" s="1">
+        <v>0.24166666666666667</v>
+      </c>
+      <c r="G9" s="1">
+        <v>6.7361111111111108E-2</v>
+      </c>
+      <c r="H9" s="1">
+        <v>0.24861111111111112</v>
+      </c>
+      <c r="I9" s="1">
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="J9" s="1">
+        <v>0.34027777777777779</v>
+      </c>
+      <c r="K9" s="1">
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="L9" s="1">
         <v>0.25833333333333336</v>
       </c>
-      <c r="G9" s="1">
+      <c r="M9" s="1">
         <v>8.2638888888888887E-2</v>
       </c>
-      <c r="H9" s="1">
+      <c r="N9" s="1">
         <v>0.25555555555555554</v>
       </c>
-      <c r="I9" s="1">
+      <c r="O9" s="1">
         <v>8.1944444444444445E-2</v>
       </c>
-      <c r="J9" s="1">
+      <c r="P9" s="1">
         <v>0.34722222222222221</v>
       </c>
-      <c r="K9" s="1">
+      <c r="Q9" s="1">
         <v>8.1944444444444445E-2</v>
-      </c>
-      <c r="L9" s="1">
-        <v>0.24166666666666667</v>
-      </c>
-      <c r="M9" s="1">
-        <v>6.7361111111111108E-2</v>
-      </c>
-      <c r="N9" s="1">
-        <v>0.24861111111111112</v>
-      </c>
-      <c r="O9" s="1">
-        <v>6.6666666666666666E-2</v>
-      </c>
-      <c r="P9" s="1">
-        <v>0.34027777777777779</v>
-      </c>
-      <c r="Q9" s="1">
-        <v>6.6666666666666666E-2</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
@@ -1165,40 +1165,40 @@
         <v>41</v>
       </c>
       <c r="F10" s="1">
+        <v>0.24305555555555555</v>
+      </c>
+      <c r="G10" s="1">
+        <v>6.8750000000000006E-2</v>
+      </c>
+      <c r="H10" s="1">
+        <v>0.24930555555555556</v>
+      </c>
+      <c r="I10" s="1">
+        <v>6.7361111111111108E-2</v>
+      </c>
+      <c r="J10" s="1">
+        <v>0.34097222222222223</v>
+      </c>
+      <c r="K10" s="1">
+        <v>6.7361111111111108E-2</v>
+      </c>
+      <c r="L10" s="1">
         <v>0.25694444444444442</v>
       </c>
-      <c r="G10" s="1">
+      <c r="M10" s="1">
         <v>8.1944444444444445E-2</v>
       </c>
-      <c r="H10" s="1">
+      <c r="N10" s="1">
         <v>0.25416666666666665</v>
       </c>
-      <c r="I10" s="1">
+      <c r="O10" s="1">
         <v>8.0555555555555561E-2</v>
       </c>
-      <c r="J10" s="1">
+      <c r="P10" s="1">
         <v>0.34583333333333333</v>
       </c>
-      <c r="K10" s="1">
+      <c r="Q10" s="1">
         <v>8.0555555555555561E-2</v>
-      </c>
-      <c r="L10" s="1">
-        <v>0.24305555555555555</v>
-      </c>
-      <c r="M10" s="1">
-        <v>6.8750000000000006E-2</v>
-      </c>
-      <c r="N10" s="1">
-        <v>0.24930555555555556</v>
-      </c>
-      <c r="O10" s="1">
-        <v>6.7361111111111108E-2</v>
-      </c>
-      <c r="P10" s="1">
-        <v>0.34097222222222223</v>
-      </c>
-      <c r="Q10" s="1">
-        <v>6.7361111111111108E-2</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -1218,40 +1218,40 @@
         <v>41</v>
       </c>
       <c r="F11" s="1">
+        <v>0.24374999999999999</v>
+      </c>
+      <c r="G11" s="1">
+        <v>6.9444444444444448E-2</v>
+      </c>
+      <c r="H11" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="I11" s="1">
+        <v>6.805555555555555E-2</v>
+      </c>
+      <c r="J11" s="1">
+        <v>0.34166666666666667</v>
+      </c>
+      <c r="K11" s="1">
+        <v>6.805555555555555E-2</v>
+      </c>
+      <c r="L11" s="1">
         <v>0.25624999999999998</v>
       </c>
-      <c r="G11" s="1">
+      <c r="M11" s="1">
         <v>8.0555555555555561E-2</v>
       </c>
-      <c r="H11" s="1">
+      <c r="N11" s="1">
         <v>0.25347222222222221</v>
       </c>
-      <c r="I11" s="1">
+      <c r="O11" s="1">
         <v>7.9861111111111105E-2</v>
       </c>
-      <c r="J11" s="1">
+      <c r="P11" s="1">
         <v>0.34513888888888888</v>
       </c>
-      <c r="K11" s="1">
+      <c r="Q11" s="1">
         <v>7.9861111111111105E-2</v>
-      </c>
-      <c r="L11" s="1">
-        <v>0.24374999999999999</v>
-      </c>
-      <c r="M11" s="1">
-        <v>6.9444444444444448E-2</v>
-      </c>
-      <c r="N11" s="1">
-        <v>0.25</v>
-      </c>
-      <c r="O11" s="1">
-        <v>6.805555555555555E-2</v>
-      </c>
-      <c r="P11" s="1">
-        <v>0.34166666666666667</v>
-      </c>
-      <c r="Q11" s="1">
-        <v>6.805555555555555E-2</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
@@ -1271,40 +1271,40 @@
         <v>14</v>
       </c>
       <c r="F12" s="1">
+        <v>0.24513888888888888</v>
+      </c>
+      <c r="G12" s="1">
+        <v>7.0833333333333331E-2</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0.25138888888888888</v>
+      </c>
+      <c r="I12" s="1">
+        <v>6.9444444444444448E-2</v>
+      </c>
+      <c r="J12" s="1">
+        <v>0.34305555555555556</v>
+      </c>
+      <c r="K12" s="1">
+        <v>6.9444444444444448E-2</v>
+      </c>
+      <c r="L12" s="1">
         <v>0.25486111111111109</v>
       </c>
-      <c r="G12" s="1">
+      <c r="M12" s="1">
         <v>7.9166666666666663E-2</v>
       </c>
-      <c r="H12" s="1">
+      <c r="N12" s="1">
         <v>0.25208333333333333</v>
       </c>
-      <c r="I12" s="1">
+      <c r="O12" s="1">
         <v>7.8472222222222221E-2</v>
       </c>
-      <c r="J12" s="1">
+      <c r="P12" s="1">
         <v>0.34375</v>
       </c>
-      <c r="K12" s="1">
+      <c r="Q12" s="1">
         <v>7.8472222222222221E-2</v>
-      </c>
-      <c r="L12" s="1">
-        <v>0.24513888888888888</v>
-      </c>
-      <c r="M12" s="1">
-        <v>7.0833333333333331E-2</v>
-      </c>
-      <c r="N12" s="1">
-        <v>0.25138888888888888</v>
-      </c>
-      <c r="O12" s="1">
-        <v>6.9444444444444448E-2</v>
-      </c>
-      <c r="P12" s="1">
-        <v>0.34305555555555556</v>
-      </c>
-      <c r="Q12" s="1">
-        <v>6.9444444444444448E-2</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
@@ -1324,40 +1324,40 @@
         <v>41</v>
       </c>
       <c r="F13" s="1">
+        <v>0.24583333333333332</v>
+      </c>
+      <c r="G13" s="1">
+        <v>7.1527777777777773E-2</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0.25208333333333333</v>
+      </c>
+      <c r="I13" s="1">
+        <v>7.013888888888889E-2</v>
+      </c>
+      <c r="J13" s="1">
+        <v>0.34375</v>
+      </c>
+      <c r="K13" s="1">
+        <v>7.013888888888889E-2</v>
+      </c>
+      <c r="L13" s="1">
         <v>0.25694444444444442</v>
       </c>
-      <c r="G13" s="1">
+      <c r="M13" s="1">
         <v>7.8472222222222221E-2</v>
       </c>
-      <c r="H13" s="1">
+      <c r="N13" s="1">
         <v>0.25069444444444444</v>
       </c>
-      <c r="I13" s="1">
+      <c r="O13" s="1">
         <v>7.7083333333333337E-2</v>
       </c>
-      <c r="J13" s="1">
+      <c r="P13" s="1">
         <v>0.34236111111111112</v>
       </c>
-      <c r="K13" s="1">
+      <c r="Q13" s="1">
         <v>7.7083333333333337E-2</v>
-      </c>
-      <c r="L13" s="1">
-        <v>0.24583333333333332</v>
-      </c>
-      <c r="M13" s="1">
-        <v>7.1527777777777773E-2</v>
-      </c>
-      <c r="N13" s="1">
-        <v>0.25208333333333333</v>
-      </c>
-      <c r="O13" s="1">
-        <v>7.013888888888889E-2</v>
-      </c>
-      <c r="P13" s="1">
-        <v>0.34375</v>
-      </c>
-      <c r="Q13" s="1">
-        <v>7.013888888888889E-2</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
@@ -1377,40 +1377,40 @@
         <v>41</v>
       </c>
       <c r="F14" s="1">
+        <v>0.24722222222222223</v>
+      </c>
+      <c r="G14" s="1">
+        <v>7.2916666666666671E-2</v>
+      </c>
+      <c r="H14" s="1">
+        <v>0.25277777777777777</v>
+      </c>
+      <c r="I14" s="1">
+        <v>7.0833333333333331E-2</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0.34444444444444444</v>
+      </c>
+      <c r="K14" s="1">
+        <v>7.0833333333333331E-2</v>
+      </c>
+      <c r="L14" s="1">
         <v>0.25555555555555554</v>
       </c>
-      <c r="G14" s="1">
+      <c r="M14" s="1">
         <v>7.7777777777777779E-2</v>
       </c>
-      <c r="H14" s="1">
+      <c r="N14" s="1">
         <v>0.25</v>
       </c>
-      <c r="I14" s="1">
+      <c r="O14" s="1">
         <v>7.6388888888888895E-2</v>
       </c>
-      <c r="J14" s="1">
+      <c r="P14" s="1">
         <v>0.34166666666666667</v>
       </c>
-      <c r="K14" s="1">
+      <c r="Q14" s="1">
         <v>7.6388888888888895E-2</v>
-      </c>
-      <c r="L14" s="1">
-        <v>0.24722222222222223</v>
-      </c>
-      <c r="M14" s="1">
-        <v>7.2916666666666671E-2</v>
-      </c>
-      <c r="N14" s="1">
-        <v>0.25277777777777777</v>
-      </c>
-      <c r="O14" s="1">
-        <v>7.0833333333333331E-2</v>
-      </c>
-      <c r="P14" s="1">
-        <v>0.34444444444444444</v>
-      </c>
-      <c r="Q14" s="1">
-        <v>7.0833333333333331E-2</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
@@ -1430,40 +1430,40 @@
         <v>41</v>
       </c>
       <c r="F15" s="1">
+        <v>0.24791666666666667</v>
+      </c>
+      <c r="G15" s="1">
+        <v>7.3611111111111113E-2</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0.25416666666666665</v>
+      </c>
+      <c r="I15" s="1">
+        <v>7.2222222222222215E-2</v>
+      </c>
+      <c r="J15" s="1">
+        <v>0.34583333333333333</v>
+      </c>
+      <c r="K15" s="1">
+        <v>7.2222222222222215E-2</v>
+      </c>
+      <c r="L15" s="1">
         <v>0.25486111111111109</v>
       </c>
-      <c r="G15" s="1">
+      <c r="M15" s="1">
         <v>7.7083333333333337E-2</v>
       </c>
-      <c r="H15" s="1">
+      <c r="N15" s="1">
         <v>0.24930555555555556</v>
       </c>
-      <c r="I15" s="1">
+      <c r="O15" s="1">
         <v>7.5694444444444439E-2</v>
       </c>
-      <c r="J15" s="1">
+      <c r="P15" s="1">
         <v>0.34097222222222223</v>
       </c>
-      <c r="K15" s="1">
+      <c r="Q15" s="1">
         <v>7.5694444444444439E-2</v>
-      </c>
-      <c r="L15" s="1">
-        <v>0.24791666666666667</v>
-      </c>
-      <c r="M15" s="1">
-        <v>7.3611111111111113E-2</v>
-      </c>
-      <c r="N15" s="1">
-        <v>0.25416666666666665</v>
-      </c>
-      <c r="O15" s="1">
-        <v>7.2222222222222215E-2</v>
-      </c>
-      <c r="P15" s="1">
-        <v>0.34583333333333333</v>
-      </c>
-      <c r="Q15" s="1">
-        <v>7.2222222222222215E-2</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
@@ -1483,40 +1483,40 @@
         <v>41</v>
       </c>
       <c r="F16" s="1">
+        <v>0.24861111111111112</v>
+      </c>
+      <c r="G16" s="1">
+        <v>7.4305555555555555E-2</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0.25486111111111109</v>
+      </c>
+      <c r="I16" s="1">
+        <v>7.2916666666666671E-2</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0.34652777777777777</v>
+      </c>
+      <c r="K16" s="1">
+        <v>7.2916666666666671E-2</v>
+      </c>
+      <c r="L16" s="1">
         <v>0.25347222222222221</v>
       </c>
-      <c r="G16" s="1">
+      <c r="M16" s="1">
         <v>7.6388888888888895E-2</v>
       </c>
-      <c r="H16" s="1">
+      <c r="N16" s="1">
         <v>0.24791666666666667</v>
       </c>
-      <c r="I16" s="1">
+      <c r="O16" s="1">
         <v>7.4305555555555555E-2</v>
       </c>
-      <c r="J16" s="1">
+      <c r="P16" s="1">
         <v>0.33958333333333335</v>
       </c>
-      <c r="K16" s="1">
+      <c r="Q16" s="1">
         <v>7.4305555555555555E-2</v>
-      </c>
-      <c r="L16" s="1">
-        <v>0.24861111111111112</v>
-      </c>
-      <c r="M16" s="1">
-        <v>7.4305555555555555E-2</v>
-      </c>
-      <c r="N16" s="1">
-        <v>0.25486111111111109</v>
-      </c>
-      <c r="O16" s="1">
-        <v>7.2916666666666671E-2</v>
-      </c>
-      <c r="P16" s="1">
-        <v>0.34652777777777777</v>
-      </c>
-      <c r="Q16" s="1">
-        <v>7.2916666666666671E-2</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.2">
@@ -1536,37 +1536,37 @@
         <v>41</v>
       </c>
       <c r="F17" s="1">
-        <v>0.25277777777777777</v>
+        <v>0.24930555555555556</v>
       </c>
       <c r="G17" s="1">
-        <v>7.4999999999999997E-2</v>
+        <v>7.5694444444444439E-2</v>
       </c>
       <c r="H17" s="1">
-        <v>0.24722222222222223</v>
+        <v>0.25555555555555554</v>
       </c>
       <c r="I17" s="1">
         <v>7.3611111111111113E-2</v>
       </c>
       <c r="J17" s="1">
-        <v>0.33819444444444446</v>
+        <v>0.34722222222222221</v>
       </c>
       <c r="K17" s="1">
         <v>7.3611111111111113E-2</v>
       </c>
       <c r="L17" s="1">
-        <v>0.24930555555555556</v>
+        <v>0.25277777777777777</v>
       </c>
       <c r="M17" s="1">
-        <v>7.5694444444444439E-2</v>
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="N17" s="1">
-        <v>0.25555555555555554</v>
+        <v>0.24722222222222223</v>
       </c>
       <c r="O17" s="1">
         <v>7.3611111111111113E-2</v>
       </c>
       <c r="P17" s="1">
-        <v>0.34722222222222221</v>
+        <v>0.33819444444444446</v>
       </c>
       <c r="Q17" s="1">
         <v>7.3611111111111113E-2</v>
@@ -1589,40 +1589,40 @@
         <v>14</v>
       </c>
       <c r="F18" s="1">
+        <v>0.25069444444444444</v>
+      </c>
+      <c r="G18" s="1">
+        <v>7.6388888888888895E-2</v>
+      </c>
+      <c r="H18" s="1">
+        <v>0.25624999999999998</v>
+      </c>
+      <c r="I18" s="1">
+        <v>7.4305555555555555E-2</v>
+      </c>
+      <c r="J18" s="1">
+        <v>0.34791666666666665</v>
+      </c>
+      <c r="K18" s="1">
+        <v>7.4305555555555555E-2</v>
+      </c>
+      <c r="L18" s="1">
         <v>0.25138888888888888</v>
       </c>
-      <c r="G18" s="1">
+      <c r="M18" s="1">
         <v>7.4305555555555555E-2</v>
       </c>
-      <c r="H18" s="1">
+      <c r="N18" s="1">
         <v>0.24652777777777779</v>
       </c>
-      <c r="I18" s="1">
+      <c r="O18" s="1">
         <v>7.2916666666666671E-2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="P18" s="1">
         <v>0.33819444444444446</v>
       </c>
-      <c r="K18" s="1">
+      <c r="Q18" s="1">
         <v>7.2916666666666671E-2</v>
-      </c>
-      <c r="L18" s="1">
-        <v>0.25069444444444444</v>
-      </c>
-      <c r="M18" s="1">
-        <v>7.6388888888888895E-2</v>
-      </c>
-      <c r="N18" s="1">
-        <v>0.25624999999999998</v>
-      </c>
-      <c r="O18" s="1">
-        <v>7.4305555555555555E-2</v>
-      </c>
-      <c r="P18" s="1">
-        <v>0.34791666666666665</v>
-      </c>
-      <c r="Q18" s="1">
-        <v>7.4305555555555555E-2</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.2">
@@ -1642,40 +1642,40 @@
         <v>41</v>
       </c>
       <c r="F19" s="1">
+        <v>0.25138888888888888</v>
+      </c>
+      <c r="G19" s="1">
+        <v>7.7777777777777779E-2</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0.25763888888888886</v>
+      </c>
+      <c r="I19" s="1">
+        <v>7.5694444444444439E-2</v>
+      </c>
+      <c r="J19" s="1">
+        <v>0.34930555555555554</v>
+      </c>
+      <c r="K19" s="1">
+        <v>7.5694444444444439E-2</v>
+      </c>
+      <c r="L19" s="1">
         <v>0.25624999999999998</v>
       </c>
-      <c r="G19" s="1">
+      <c r="M19" s="1">
         <v>7.2916666666666671E-2</v>
       </c>
-      <c r="H19" s="1">
+      <c r="N19" s="1">
         <v>0.24930555555555556</v>
       </c>
-      <c r="I19" s="1">
+      <c r="O19" s="1">
         <v>7.1527777777777773E-2</v>
       </c>
-      <c r="J19" s="1">
+      <c r="P19" s="1">
         <v>0.33680555555555558</v>
       </c>
-      <c r="K19" s="1">
+      <c r="Q19" s="1">
         <v>7.1527777777777773E-2</v>
-      </c>
-      <c r="L19" s="1">
-        <v>0.25138888888888888</v>
-      </c>
-      <c r="M19" s="1">
-        <v>7.7777777777777779E-2</v>
-      </c>
-      <c r="N19" s="1">
-        <v>0.25763888888888886</v>
-      </c>
-      <c r="O19" s="1">
-        <v>7.5694444444444439E-2</v>
-      </c>
-      <c r="P19" s="1">
-        <v>0.34930555555555554</v>
-      </c>
-      <c r="Q19" s="1">
-        <v>7.5694444444444439E-2</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.2">
@@ -1695,40 +1695,40 @@
         <v>41</v>
       </c>
       <c r="F20" s="1">
+        <v>0.25277777777777777</v>
+      </c>
+      <c r="G20" s="1">
+        <v>7.8472222222222221E-2</v>
+      </c>
+      <c r="H20" s="1">
+        <v>0.25833333333333336</v>
+      </c>
+      <c r="I20" s="1">
+        <v>7.6388888888888895E-2</v>
+      </c>
+      <c r="J20" s="1">
+        <v>0.35</v>
+      </c>
+      <c r="K20" s="1">
+        <v>7.6388888888888895E-2</v>
+      </c>
+      <c r="L20" s="1">
         <v>0.25486111111111109</v>
       </c>
-      <c r="G20" s="1">
+      <c r="M20" s="1">
         <v>7.2222222222222215E-2</v>
       </c>
-      <c r="H20" s="1">
+      <c r="N20" s="1">
         <v>0.24861111111111112</v>
       </c>
-      <c r="I20" s="1">
+      <c r="O20" s="1">
         <v>7.0833333333333331E-2</v>
       </c>
-      <c r="J20" s="1">
+      <c r="P20" s="1">
         <v>0.33611111111111114</v>
       </c>
-      <c r="K20" s="1">
+      <c r="Q20" s="1">
         <v>7.0833333333333331E-2</v>
-      </c>
-      <c r="L20" s="1">
-        <v>0.25277777777777777</v>
-      </c>
-      <c r="M20" s="1">
-        <v>7.8472222222222221E-2</v>
-      </c>
-      <c r="N20" s="1">
-        <v>0.25833333333333336</v>
-      </c>
-      <c r="O20" s="1">
-        <v>7.6388888888888895E-2</v>
-      </c>
-      <c r="P20" s="1">
-        <v>0.35</v>
-      </c>
-      <c r="Q20" s="1">
-        <v>7.6388888888888895E-2</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.2">
@@ -1748,40 +1748,40 @@
         <v>41</v>
       </c>
       <c r="F21" s="1">
+        <v>0.25486111111111109</v>
+      </c>
+      <c r="G21" s="1">
+        <v>8.0555555555555561E-2</v>
+      </c>
+      <c r="H21" s="1">
+        <v>0.25972222222222224</v>
+      </c>
+      <c r="I21" s="1">
+        <v>7.7777777777777779E-2</v>
+      </c>
+      <c r="J21" s="1">
+        <v>0.35138888888888886</v>
+      </c>
+      <c r="K21" s="1">
+        <v>7.7777777777777779E-2</v>
+      </c>
+      <c r="L21" s="1">
         <v>0.25277777777777777</v>
       </c>
-      <c r="G21" s="1">
+      <c r="M21" s="1">
         <v>7.013888888888889E-2</v>
       </c>
-      <c r="H21" s="1">
+      <c r="N21" s="1">
         <v>0.25138888888888888</v>
       </c>
-      <c r="I21" s="1">
+      <c r="O21" s="1">
         <v>6.9444444444444448E-2</v>
       </c>
-      <c r="J21" s="1">
+      <c r="P21" s="1">
         <v>0.3347222222222222</v>
       </c>
-      <c r="K21" s="1">
+      <c r="Q21" s="1">
         <v>6.9444444444444448E-2</v>
-      </c>
-      <c r="L21" s="1">
-        <v>0.25486111111111109</v>
-      </c>
-      <c r="M21" s="1">
-        <v>8.0555555555555561E-2</v>
-      </c>
-      <c r="N21" s="1">
-        <v>0.25972222222222224</v>
-      </c>
-      <c r="O21" s="1">
-        <v>7.7777777777777779E-2</v>
-      </c>
-      <c r="P21" s="1">
-        <v>0.35138888888888886</v>
-      </c>
-      <c r="Q21" s="1">
-        <v>7.7777777777777779E-2</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.2">
@@ -1801,40 +1801,40 @@
         <v>41</v>
       </c>
       <c r="F22" s="1">
+        <v>0.25624999999999998</v>
+      </c>
+      <c r="G22" s="1">
+        <v>8.1944444444444445E-2</v>
+      </c>
+      <c r="H22" s="1">
+        <v>0.26111111111111113</v>
+      </c>
+      <c r="I22" s="1">
+        <v>7.9166666666666663E-2</v>
+      </c>
+      <c r="J22" s="1">
+        <v>0.3527777777777778</v>
+      </c>
+      <c r="K22" s="1">
+        <v>7.9166666666666663E-2</v>
+      </c>
+      <c r="L22" s="1">
         <v>0.25138888888888888</v>
       </c>
-      <c r="G22" s="1">
+      <c r="M22" s="1">
         <v>6.8750000000000006E-2</v>
       </c>
-      <c r="H22" s="1">
+      <c r="N22" s="1">
         <v>0.25</v>
       </c>
-      <c r="I22" s="1">
+      <c r="O22" s="1">
         <v>6.805555555555555E-2</v>
       </c>
-      <c r="J22" s="1">
+      <c r="P22" s="1">
         <v>0.33333333333333331</v>
       </c>
-      <c r="K22" s="1">
+      <c r="Q22" s="1">
         <v>6.805555555555555E-2</v>
-      </c>
-      <c r="L22" s="1">
-        <v>0.25624999999999998</v>
-      </c>
-      <c r="M22" s="1">
-        <v>8.1944444444444445E-2</v>
-      </c>
-      <c r="N22" s="1">
-        <v>0.26111111111111113</v>
-      </c>
-      <c r="O22" s="1">
-        <v>7.9166666666666663E-2</v>
-      </c>
-      <c r="P22" s="1">
-        <v>0.3527777777777778</v>
-      </c>
-      <c r="Q22" s="1">
-        <v>7.9166666666666663E-2</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.2">
@@ -1854,40 +1854,40 @@
         <v>14</v>
       </c>
       <c r="F23" s="1">
+        <v>0.25694444444444442</v>
+      </c>
+      <c r="G23" s="1">
+        <v>8.2638888888888887E-2</v>
+      </c>
+      <c r="H23" s="1">
+        <v>0.26180555555555557</v>
+      </c>
+      <c r="I23" s="1">
+        <v>7.9861111111111105E-2</v>
+      </c>
+      <c r="J23" s="1">
+        <v>0.35347222222222224</v>
+      </c>
+      <c r="K23" s="1">
+        <v>7.9861111111111105E-2</v>
+      </c>
+      <c r="L23" s="1">
         <v>0.25069444444444444</v>
       </c>
-      <c r="G23" s="1">
+      <c r="M23" s="1">
         <v>6.805555555555555E-2</v>
       </c>
-      <c r="H23" s="1">
+      <c r="N23" s="1">
         <v>0.24861111111111112</v>
       </c>
-      <c r="I23" s="1">
+      <c r="O23" s="1">
         <v>6.6666666666666666E-2</v>
       </c>
-      <c r="J23" s="1">
+      <c r="P23" s="1">
         <v>0.33194444444444443</v>
       </c>
-      <c r="K23" s="1">
+      <c r="Q23" s="1">
         <v>6.6666666666666666E-2</v>
-      </c>
-      <c r="L23" s="1">
-        <v>0.25694444444444442</v>
-      </c>
-      <c r="M23" s="1">
-        <v>8.2638888888888887E-2</v>
-      </c>
-      <c r="N23" s="1">
-        <v>0.26180555555555557</v>
-      </c>
-      <c r="O23" s="1">
-        <v>7.9861111111111105E-2</v>
-      </c>
-      <c r="P23" s="1">
-        <v>0.35347222222222224</v>
-      </c>
-      <c r="Q23" s="1">
-        <v>7.9861111111111105E-2</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.2">
@@ -1907,40 +1907,40 @@
         <v>14</v>
       </c>
       <c r="F24" s="1">
+        <v>0.25833333333333336</v>
+      </c>
+      <c r="G24" s="1">
+        <v>8.4027777777777785E-2</v>
+      </c>
+      <c r="H24" s="1">
+        <v>0.26319444444444445</v>
+      </c>
+      <c r="I24" s="1">
+        <v>8.1250000000000003E-2</v>
+      </c>
+      <c r="J24" s="1">
+        <v>0.35486111111111113</v>
+      </c>
+      <c r="K24" s="1">
+        <v>8.1250000000000003E-2</v>
+      </c>
+      <c r="L24" s="1">
         <v>0.25416666666666665</v>
       </c>
-      <c r="G24" s="1">
+      <c r="M24" s="1">
         <v>6.6666666666666666E-2</v>
       </c>
-      <c r="H24" s="1">
+      <c r="N24" s="1">
         <v>0.25208333333333333</v>
       </c>
-      <c r="I24" s="1">
+      <c r="O24" s="1">
         <v>6.5972222222222224E-2</v>
       </c>
-      <c r="J24" s="1">
+      <c r="P24" s="1">
         <v>0.33124999999999999</v>
       </c>
-      <c r="K24" s="1">
+      <c r="Q24" s="1">
         <v>6.5972222222222224E-2</v>
-      </c>
-      <c r="L24" s="1">
-        <v>0.25833333333333336</v>
-      </c>
-      <c r="M24" s="1">
-        <v>8.4027777777777785E-2</v>
-      </c>
-      <c r="N24" s="1">
-        <v>0.26319444444444445</v>
-      </c>
-      <c r="O24" s="1">
-        <v>8.1250000000000003E-2</v>
-      </c>
-      <c r="P24" s="1">
-        <v>0.35486111111111113</v>
-      </c>
-      <c r="Q24" s="1">
-        <v>8.1250000000000003E-2</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.2">
@@ -1960,40 +1960,40 @@
         <v>41</v>
       </c>
       <c r="F25" s="1">
+        <v>0.2590277777777778</v>
+      </c>
+      <c r="G25" s="1">
+        <v>8.4722222222222227E-2</v>
+      </c>
+      <c r="H25" s="1">
+        <v>0.2638888888888889</v>
+      </c>
+      <c r="I25" s="1">
+        <v>8.1944444444444445E-2</v>
+      </c>
+      <c r="J25" s="1">
+        <v>0.35555555555555557</v>
+      </c>
+      <c r="K25" s="1">
+        <v>8.1944444444444445E-2</v>
+      </c>
+      <c r="L25" s="1">
         <v>0.25347222222222221</v>
       </c>
-      <c r="G25" s="1">
+      <c r="M25" s="1">
         <v>6.5972222222222224E-2</v>
       </c>
-      <c r="H25" s="1">
+      <c r="N25" s="1">
         <v>0.25138888888888888</v>
       </c>
-      <c r="I25" s="1">
+      <c r="O25" s="1">
         <v>6.5972222222222224E-2</v>
       </c>
-      <c r="J25" s="1">
+      <c r="P25" s="1">
         <v>0.33055555555555555</v>
       </c>
-      <c r="K25" s="1">
+      <c r="Q25" s="1">
         <v>6.5277777777777782E-2</v>
-      </c>
-      <c r="L25" s="1">
-        <v>0.2590277777777778</v>
-      </c>
-      <c r="M25" s="1">
-        <v>8.4722222222222227E-2</v>
-      </c>
-      <c r="N25" s="1">
-        <v>0.2638888888888889</v>
-      </c>
-      <c r="O25" s="1">
-        <v>8.1944444444444445E-2</v>
-      </c>
-      <c r="P25" s="1">
-        <v>0.35555555555555557</v>
-      </c>
-      <c r="Q25" s="1">
-        <v>8.1944444444444445E-2</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.2">
@@ -2013,40 +2013,40 @@
         <v>41</v>
       </c>
       <c r="F26" s="1">
+        <v>0.26111111111111113</v>
+      </c>
+      <c r="G26" s="1">
+        <v>8.6805555555555552E-2</v>
+      </c>
+      <c r="H26" s="1">
+        <v>0.26597222222222222</v>
+      </c>
+      <c r="I26" s="1">
+        <v>8.4027777777777785E-2</v>
+      </c>
+      <c r="J26" s="1">
+        <v>0.3576388888888889</v>
+      </c>
+      <c r="K26" s="1">
+        <v>8.4027777777777785E-2</v>
+      </c>
+      <c r="L26" s="1">
         <v>0.25138888888888888</v>
       </c>
-      <c r="G26" s="1">
+      <c r="M26" s="1">
         <v>6.3888888888888884E-2</v>
       </c>
-      <c r="H26" s="1">
+      <c r="N26" s="1">
         <v>0.24930555555555556</v>
       </c>
-      <c r="I26" s="1">
+      <c r="O26" s="1">
         <v>6.3194444444444442E-2</v>
       </c>
-      <c r="J26" s="1">
+      <c r="P26" s="1">
         <v>0.32847222222222222</v>
       </c>
-      <c r="K26" s="1">
+      <c r="Q26" s="1">
         <v>6.3194444444444442E-2</v>
-      </c>
-      <c r="L26" s="1">
-        <v>0.26111111111111113</v>
-      </c>
-      <c r="M26" s="1">
-        <v>8.6805555555555552E-2</v>
-      </c>
-      <c r="N26" s="1">
-        <v>0.26597222222222222</v>
-      </c>
-      <c r="O26" s="1">
-        <v>8.4027777777777785E-2</v>
-      </c>
-      <c r="P26" s="1">
-        <v>0.3576388888888889</v>
-      </c>
-      <c r="Q26" s="1">
-        <v>8.4027777777777785E-2</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.2">
@@ -2066,40 +2066,40 @@
         <v>41</v>
       </c>
       <c r="F27" s="1">
+        <v>0.26458333333333334</v>
+      </c>
+      <c r="G27" s="1">
+        <v>9.0277777777777776E-2</v>
+      </c>
+      <c r="H27" s="1">
+        <v>0.26874999999999999</v>
+      </c>
+      <c r="I27" s="1">
+        <v>8.6805555555555552E-2</v>
+      </c>
+      <c r="J27" s="1">
+        <v>0.36041666666666666</v>
+      </c>
+      <c r="K27" s="1">
+        <v>8.6805555555555552E-2</v>
+      </c>
+      <c r="L27" s="1">
         <v>0.25277777777777777</v>
       </c>
-      <c r="G27" s="1">
+      <c r="M27" s="1">
         <v>6.1111111111111109E-2</v>
       </c>
-      <c r="H27" s="1">
+      <c r="N27" s="1">
         <v>0.25</v>
       </c>
-      <c r="I27" s="1">
+      <c r="O27" s="1">
         <v>5.9722222222222225E-2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="P27" s="1">
         <v>0.32500000000000001</v>
       </c>
-      <c r="K27" s="1">
+      <c r="Q27" s="1">
         <v>5.9722222222222225E-2</v>
-      </c>
-      <c r="L27" s="1">
-        <v>0.26458333333333334</v>
-      </c>
-      <c r="M27" s="1">
-        <v>9.0277777777777776E-2</v>
-      </c>
-      <c r="N27" s="1">
-        <v>0.26874999999999999</v>
-      </c>
-      <c r="O27" s="1">
-        <v>8.6805555555555552E-2</v>
-      </c>
-      <c r="P27" s="1">
-        <v>0.36041666666666666</v>
-      </c>
-      <c r="Q27" s="1">
-        <v>8.6805555555555552E-2</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.2">
@@ -2119,40 +2119,40 @@
         <v>41</v>
       </c>
       <c r="F28" s="1">
+        <v>0.26527777777777778</v>
+      </c>
+      <c r="G28" s="1">
+        <v>9.0972222222222218E-2</v>
+      </c>
+      <c r="H28" s="1">
+        <v>0.27013888888888887</v>
+      </c>
+      <c r="I28" s="1">
+        <v>8.819444444444445E-2</v>
+      </c>
+      <c r="J28" s="1">
+        <v>0.36180555555555555</v>
+      </c>
+      <c r="K28" s="1">
+        <v>8.819444444444445E-2</v>
+      </c>
+      <c r="L28" s="1">
         <v>0.25138888888888888</v>
       </c>
-      <c r="G28" s="1">
+      <c r="M28" s="1">
         <v>5.9722222222222225E-2</v>
       </c>
-      <c r="H28" s="1">
+      <c r="N28" s="1">
         <v>0.24930555555555556</v>
       </c>
-      <c r="I28" s="1">
+      <c r="O28" s="1">
         <v>5.9027777777777776E-2</v>
       </c>
-      <c r="J28" s="1">
+      <c r="P28" s="1">
         <v>0.32430555555555557</v>
       </c>
-      <c r="K28" s="1">
+      <c r="Q28" s="1">
         <v>5.9027777777777776E-2</v>
-      </c>
-      <c r="L28" s="1">
-        <v>0.26527777777777778</v>
-      </c>
-      <c r="M28" s="1">
-        <v>9.0972222222222218E-2</v>
-      </c>
-      <c r="N28" s="1">
-        <v>0.27013888888888887</v>
-      </c>
-      <c r="O28" s="1">
-        <v>8.819444444444445E-2</v>
-      </c>
-      <c r="P28" s="1">
-        <v>0.36180555555555555</v>
-      </c>
-      <c r="Q28" s="1">
-        <v>8.819444444444445E-2</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.2">
@@ -2172,40 +2172,40 @@
         <v>41</v>
       </c>
       <c r="F29" s="1">
+        <v>0.26666666666666666</v>
+      </c>
+      <c r="G29" s="1">
+        <v>9.2361111111111116E-2</v>
+      </c>
+      <c r="H29" s="1">
+        <v>0.27083333333333331</v>
+      </c>
+      <c r="I29" s="1">
+        <v>8.8888888888888892E-2</v>
+      </c>
+      <c r="J29" s="1">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="K29" s="1">
+        <v>8.8888888888888892E-2</v>
+      </c>
+      <c r="L29" s="1">
         <v>0.25</v>
       </c>
-      <c r="G29" s="1">
+      <c r="M29" s="1">
         <v>5.9027777777777776E-2</v>
       </c>
-      <c r="H29" s="1">
+      <c r="N29" s="1">
         <v>0.24791666666666667</v>
       </c>
-      <c r="I29" s="1">
+      <c r="O29" s="1">
         <v>5.7638888888888892E-2</v>
       </c>
-      <c r="J29" s="1">
+      <c r="P29" s="1">
         <v>0.32291666666666669</v>
       </c>
-      <c r="K29" s="1">
+      <c r="Q29" s="1">
         <v>5.7638888888888892E-2</v>
-      </c>
-      <c r="L29" s="1">
-        <v>0.26666666666666666</v>
-      </c>
-      <c r="M29" s="1">
-        <v>9.2361111111111116E-2</v>
-      </c>
-      <c r="N29" s="1">
-        <v>0.27083333333333331</v>
-      </c>
-      <c r="O29" s="1">
-        <v>8.8888888888888892E-2</v>
-      </c>
-      <c r="P29" s="1">
-        <v>0.36249999999999999</v>
-      </c>
-      <c r="Q29" s="1">
-        <v>8.8888888888888892E-2</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.2">
@@ -2225,40 +2225,40 @@
         <v>41</v>
       </c>
       <c r="F30" s="1">
+        <v>0.26805555555555555</v>
+      </c>
+      <c r="G30" s="1">
+        <v>9.4444444444444442E-2</v>
+      </c>
+      <c r="H30" s="1">
+        <v>0.2722222222222222</v>
+      </c>
+      <c r="I30" s="1">
+        <v>9.0277777777777776E-2</v>
+      </c>
+      <c r="J30" s="1">
+        <v>0.36388888888888887</v>
+      </c>
+      <c r="K30" s="1">
+        <v>9.0277777777777776E-2</v>
+      </c>
+      <c r="L30" s="1">
         <v>0.24861111111111112</v>
       </c>
-      <c r="G30" s="1">
+      <c r="M30" s="1">
         <v>5.7638888888888892E-2</v>
       </c>
-      <c r="H30" s="1">
+      <c r="N30" s="1">
         <v>0.24722222222222223</v>
       </c>
-      <c r="I30" s="1">
+      <c r="O30" s="1">
         <v>5.6944444444444443E-2</v>
       </c>
-      <c r="J30" s="1">
+      <c r="P30" s="1">
         <v>0.32222222222222224</v>
       </c>
-      <c r="K30" s="1">
+      <c r="Q30" s="1">
         <v>5.6944444444444443E-2</v>
-      </c>
-      <c r="L30" s="1">
-        <v>0.26805555555555555</v>
-      </c>
-      <c r="M30" s="1">
-        <v>9.4444444444444442E-2</v>
-      </c>
-      <c r="N30" s="1">
-        <v>0.2722222222222222</v>
-      </c>
-      <c r="O30" s="1">
-        <v>9.0277777777777776E-2</v>
-      </c>
-      <c r="P30" s="1">
-        <v>0.36388888888888887</v>
-      </c>
-      <c r="Q30" s="1">
-        <v>9.0277777777777776E-2</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.2">
@@ -2278,40 +2278,40 @@
         <v>41</v>
       </c>
       <c r="F31" s="1">
+        <v>0.26944444444444443</v>
+      </c>
+      <c r="G31" s="1">
+        <v>9.583333333333334E-2</v>
+      </c>
+      <c r="H31" s="1">
+        <v>0.27361111111111114</v>
+      </c>
+      <c r="I31" s="1">
+        <v>9.166666666666666E-2</v>
+      </c>
+      <c r="J31" s="1">
+        <v>0.36527777777777776</v>
+      </c>
+      <c r="K31" s="1">
+        <v>9.166666666666666E-2</v>
+      </c>
+      <c r="L31" s="1">
         <v>0.24722222222222223</v>
       </c>
-      <c r="G31" s="1">
+      <c r="M31" s="1">
         <v>5.6250000000000001E-2</v>
       </c>
-      <c r="H31" s="1">
+      <c r="N31" s="1">
         <v>0.24583333333333332</v>
       </c>
-      <c r="I31" s="1">
+      <c r="O31" s="1">
         <v>5.5555555555555552E-2</v>
       </c>
-      <c r="J31" s="1">
+      <c r="P31" s="1">
         <v>0.32083333333333336</v>
       </c>
-      <c r="K31" s="1">
+      <c r="Q31" s="1">
         <v>5.5555555555555552E-2</v>
-      </c>
-      <c r="L31" s="1">
-        <v>0.26944444444444443</v>
-      </c>
-      <c r="M31" s="1">
-        <v>9.583333333333334E-2</v>
-      </c>
-      <c r="N31" s="1">
-        <v>0.27361111111111114</v>
-      </c>
-      <c r="O31" s="1">
-        <v>9.166666666666666E-2</v>
-      </c>
-      <c r="P31" s="1">
-        <v>0.36527777777777776</v>
-      </c>
-      <c r="Q31" s="1">
-        <v>9.166666666666666E-2</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.2">
@@ -2331,40 +2331,40 @@
         <v>41</v>
       </c>
       <c r="F32" s="1">
+        <v>0.24027777777777778</v>
+      </c>
+      <c r="G32" s="1">
+        <v>9.8611111111111108E-2</v>
+      </c>
+      <c r="H32" s="1">
+        <v>0.24791666666666667</v>
+      </c>
+      <c r="I32" s="1">
+        <v>9.5138888888888884E-2</v>
+      </c>
+      <c r="J32" s="1">
+        <v>0.32291666666666669</v>
+      </c>
+      <c r="K32" s="1">
+        <v>9.5138888888888884E-2</v>
+      </c>
+      <c r="L32" s="1">
         <v>0.25347222222222221</v>
       </c>
-      <c r="G32" s="1">
+      <c r="M32" s="1">
         <v>6.6666666666666666E-2</v>
       </c>
-      <c r="H32" s="1">
+      <c r="N32" s="1">
         <v>0.25208333333333333</v>
       </c>
-      <c r="I32" s="1">
+      <c r="O32" s="1">
         <v>6.5972222222222224E-2</v>
       </c>
-      <c r="J32" s="1">
+      <c r="P32" s="1">
         <v>0.33541666666666664</v>
       </c>
-      <c r="K32" s="1">
+      <c r="Q32" s="1">
         <v>6.5972222222222224E-2</v>
-      </c>
-      <c r="L32" s="1">
-        <v>0.24027777777777778</v>
-      </c>
-      <c r="M32" s="1">
-        <v>9.8611111111111108E-2</v>
-      </c>
-      <c r="N32" s="1">
-        <v>0.24791666666666667</v>
-      </c>
-      <c r="O32" s="1">
-        <v>9.5138888888888884E-2</v>
-      </c>
-      <c r="P32" s="1">
-        <v>0.32291666666666669</v>
-      </c>
-      <c r="Q32" s="1">
-        <v>9.5138888888888884E-2</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.2">
@@ -2384,40 +2384,40 @@
         <v>41</v>
       </c>
       <c r="F33" s="1">
+        <v>0.24166666666666667</v>
+      </c>
+      <c r="G33" s="1">
+        <v>0.10069444444444445</v>
+      </c>
+      <c r="H33" s="1">
+        <v>0.24930555555555556</v>
+      </c>
+      <c r="I33" s="1">
+        <v>9.6527777777777782E-2</v>
+      </c>
+      <c r="J33" s="1">
+        <v>0.32430555555555557</v>
+      </c>
+      <c r="K33" s="1">
+        <v>9.6527777777777782E-2</v>
+      </c>
+      <c r="L33" s="1">
         <v>0.25138888888888888</v>
       </c>
-      <c r="G33" s="1">
+      <c r="M33" s="1">
         <v>6.5277777777777782E-2</v>
       </c>
-      <c r="H33" s="1">
+      <c r="N33" s="1">
         <v>0.25</v>
       </c>
-      <c r="I33" s="1">
+      <c r="O33" s="1">
         <v>6.3888888888888884E-2</v>
       </c>
-      <c r="J33" s="1">
+      <c r="P33" s="1">
         <v>0.33333333333333331</v>
       </c>
-      <c r="K33" s="1">
+      <c r="Q33" s="1">
         <v>6.3888888888888884E-2</v>
-      </c>
-      <c r="L33" s="1">
-        <v>0.24166666666666667</v>
-      </c>
-      <c r="M33" s="1">
-        <v>0.10069444444444445</v>
-      </c>
-      <c r="N33" s="1">
-        <v>0.24930555555555556</v>
-      </c>
-      <c r="O33" s="1">
-        <v>9.6527777777777782E-2</v>
-      </c>
-      <c r="P33" s="1">
-        <v>0.32430555555555557</v>
-      </c>
-      <c r="Q33" s="1">
-        <v>9.6527777777777782E-2</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.2">
@@ -2437,40 +2437,40 @@
         <v>41</v>
       </c>
       <c r="F34" s="1">
+        <v>0.24374999999999999</v>
+      </c>
+      <c r="G34" s="1">
+        <v>0.10208333333333333</v>
+      </c>
+      <c r="H34" s="1">
+        <v>0.25138888888888888</v>
+      </c>
+      <c r="I34" s="1">
+        <v>9.8611111111111108E-2</v>
+      </c>
+      <c r="J34" s="1">
+        <v>0.3263888888888889</v>
+      </c>
+      <c r="K34" s="1">
+        <v>9.8611111111111108E-2</v>
+      </c>
+      <c r="L34" s="1">
         <v>0.25</v>
       </c>
-      <c r="G34" s="1">
+      <c r="M34" s="1">
         <v>6.3194444444444442E-2</v>
       </c>
-      <c r="H34" s="1">
+      <c r="N34" s="1">
         <v>0.24861111111111112</v>
       </c>
-      <c r="I34" s="1">
+      <c r="O34" s="1">
         <v>6.25E-2</v>
       </c>
-      <c r="J34" s="1">
+      <c r="P34" s="1">
         <v>0.33194444444444443</v>
       </c>
-      <c r="K34" s="1">
+      <c r="Q34" s="1">
         <v>6.25E-2</v>
-      </c>
-      <c r="L34" s="1">
-        <v>0.24374999999999999</v>
-      </c>
-      <c r="M34" s="1">
-        <v>0.10208333333333333</v>
-      </c>
-      <c r="N34" s="1">
-        <v>0.25138888888888888</v>
-      </c>
-      <c r="O34" s="1">
-        <v>9.8611111111111108E-2</v>
-      </c>
-      <c r="P34" s="1">
-        <v>0.3263888888888889</v>
-      </c>
-      <c r="Q34" s="1">
-        <v>9.8611111111111108E-2</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.2">
@@ -2490,40 +2490,40 @@
         <v>41</v>
       </c>
       <c r="F35" s="1">
+        <v>0.24513888888888888</v>
+      </c>
+      <c r="G35" s="1">
+        <v>0.10416666666666667</v>
+      </c>
+      <c r="H35" s="1">
+        <v>0.25277777777777777</v>
+      </c>
+      <c r="I35" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="J35" s="1">
+        <v>0.32777777777777778</v>
+      </c>
+      <c r="K35" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="L35" s="1">
         <v>0.24791666666666667</v>
       </c>
-      <c r="G35" s="1">
+      <c r="M35" s="1">
         <v>6.1805555555555558E-2</v>
       </c>
-      <c r="H35" s="1">
+      <c r="N35" s="1">
         <v>0.24652777777777779</v>
       </c>
-      <c r="I35" s="1">
+      <c r="O35" s="1">
         <v>6.0416666666666667E-2</v>
       </c>
-      <c r="J35" s="1">
+      <c r="P35" s="1">
         <v>0.3298611111111111</v>
       </c>
-      <c r="K35" s="1">
+      <c r="Q35" s="1">
         <v>6.0416666666666667E-2</v>
-      </c>
-      <c r="L35" s="1">
-        <v>0.24513888888888888</v>
-      </c>
-      <c r="M35" s="1">
-        <v>0.10416666666666667</v>
-      </c>
-      <c r="N35" s="1">
-        <v>0.25277777777777777</v>
-      </c>
-      <c r="O35" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="P35" s="1">
-        <v>0.32777777777777778</v>
-      </c>
-      <c r="Q35" s="1">
-        <v>0.1</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.2">
@@ -2546,37 +2546,37 @@
         <v>0.24652777777777779</v>
       </c>
       <c r="G36" s="1">
-        <v>6.0416666666666667E-2</v>
+        <v>0.10486111111111111</v>
       </c>
       <c r="H36" s="1">
-        <v>0.24583333333333332</v>
+        <v>0.25416666666666665</v>
       </c>
       <c r="I36" s="1">
-        <v>5.9722222222222225E-2</v>
+        <v>0.10138888888888889</v>
       </c>
       <c r="J36" s="1">
         <v>0.32916666666666666</v>
       </c>
       <c r="K36" s="1">
-        <v>5.9722222222222225E-2</v>
+        <v>0.10138888888888889</v>
       </c>
       <c r="L36" s="1">
         <v>0.24652777777777779</v>
       </c>
       <c r="M36" s="1">
-        <v>0.10486111111111111</v>
+        <v>6.0416666666666667E-2</v>
       </c>
       <c r="N36" s="1">
-        <v>0.25416666666666665</v>
+        <v>0.24583333333333332</v>
       </c>
       <c r="O36" s="1">
-        <v>0.10138888888888889</v>
+        <v>5.9722222222222225E-2</v>
       </c>
       <c r="P36" s="1">
         <v>0.32916666666666666</v>
       </c>
       <c r="Q36" s="1">
-        <v>0.10138888888888889</v>
+        <v>5.9722222222222225E-2</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.2">
@@ -2596,40 +2596,40 @@
         <v>41</v>
       </c>
       <c r="F37" s="1">
+        <v>0.24791666666666667</v>
+      </c>
+      <c r="G37" s="1">
+        <v>0.10625</v>
+      </c>
+      <c r="H37" s="1">
+        <v>0.25555555555555554</v>
+      </c>
+      <c r="I37" s="1">
+        <v>0.10277777777777777</v>
+      </c>
+      <c r="J37" s="1">
+        <v>0.33055555555555555</v>
+      </c>
+      <c r="K37" s="1">
+        <v>0.10277777777777777</v>
+      </c>
+      <c r="L37" s="1">
         <v>0.24513888888888888</v>
       </c>
-      <c r="G37" s="1">
+      <c r="M37" s="1">
         <v>5.9027777777777776E-2</v>
       </c>
-      <c r="H37" s="1">
+      <c r="N37" s="1">
         <v>0.24444444444444444</v>
       </c>
-      <c r="I37" s="1">
+      <c r="O37" s="1">
         <v>5.8333333333333334E-2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="P37" s="1">
         <v>0.32777777777777778</v>
       </c>
-      <c r="K37" s="1">
+      <c r="Q37" s="1">
         <v>5.8333333333333334E-2</v>
-      </c>
-      <c r="L37" s="1">
-        <v>0.24791666666666667</v>
-      </c>
-      <c r="M37" s="1">
-        <v>0.10625</v>
-      </c>
-      <c r="N37" s="1">
-        <v>0.25555555555555554</v>
-      </c>
-      <c r="O37" s="1">
-        <v>0.10277777777777777</v>
-      </c>
-      <c r="P37" s="1">
-        <v>0.33055555555555555</v>
-      </c>
-      <c r="Q37" s="1">
-        <v>0.10277777777777777</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.2">
@@ -2649,40 +2649,40 @@
         <v>14</v>
       </c>
       <c r="F38" s="1">
+        <v>0.24930555555555556</v>
+      </c>
+      <c r="G38" s="1">
+        <v>0.1076388888888889</v>
+      </c>
+      <c r="H38" s="1">
+        <v>0.25694444444444442</v>
+      </c>
+      <c r="I38" s="1">
+        <v>0.10416666666666667</v>
+      </c>
+      <c r="J38" s="1">
+        <v>0.33194444444444443</v>
+      </c>
+      <c r="K38" s="1">
+        <v>0.10416666666666667</v>
+      </c>
+      <c r="L38" s="1">
         <v>0.24374999999999999</v>
       </c>
-      <c r="G38" s="1">
+      <c r="M38" s="1">
         <v>5.7638888888888892E-2</v>
       </c>
-      <c r="H38" s="1">
+      <c r="N38" s="1">
         <v>0.24305555555555555</v>
       </c>
-      <c r="I38" s="1">
+      <c r="O38" s="1">
         <v>5.6944444444444443E-2</v>
       </c>
-      <c r="J38" s="1">
+      <c r="P38" s="1">
         <v>0.3263888888888889</v>
       </c>
-      <c r="K38" s="1">
+      <c r="Q38" s="1">
         <v>5.6944444444444443E-2</v>
-      </c>
-      <c r="L38" s="1">
-        <v>0.24930555555555556</v>
-      </c>
-      <c r="M38" s="1">
-        <v>0.1076388888888889</v>
-      </c>
-      <c r="N38" s="1">
-        <v>0.25694444444444442</v>
-      </c>
-      <c r="O38" s="1">
-        <v>0.10416666666666667</v>
-      </c>
-      <c r="P38" s="1">
-        <v>0.33194444444444443</v>
-      </c>
-      <c r="Q38" s="1">
-        <v>0.10416666666666667</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.2">
@@ -2695,6 +2695,48 @@
       <c r="C39" t="s">
         <v>56</v>
       </c>
+      <c r="D39" t="s">
+        <v>14</v>
+      </c>
+      <c r="E39" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39" s="1">
+        <v>0.2361111111111111</v>
+      </c>
+      <c r="G39" s="1">
+        <v>6.3194444444444442E-2</v>
+      </c>
+      <c r="H39" s="1">
+        <v>0.24166666666666667</v>
+      </c>
+      <c r="I39" s="1">
+        <v>6.1805555555555558E-2</v>
+      </c>
+      <c r="J39" s="1">
+        <v>0.33263888888888887</v>
+      </c>
+      <c r="K39" s="1">
+        <v>6.1805555555555558E-2</v>
+      </c>
+      <c r="L39" s="1">
+        <v>0.24722222222222223</v>
+      </c>
+      <c r="M39" s="1">
+        <v>9.4444444444444442E-2</v>
+      </c>
+      <c r="N39" s="1">
+        <v>0.25069444444444444</v>
+      </c>
+      <c r="O39" s="1">
+        <v>9.583333333333334E-2</v>
+      </c>
+      <c r="P39" s="1">
+        <v>0.34375</v>
+      </c>
+      <c r="Q39" s="1">
+        <v>9.583333333333334E-2</v>
+      </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A40">
@@ -2706,6 +2748,50 @@
       <c r="C40" t="s">
         <v>57</v>
       </c>
+      <c r="F40" s="1">
+        <v>0.23749999999999999</v>
+      </c>
+      <c r="G40" s="1">
+        <v>6.458333333333334E-2</v>
+      </c>
+      <c r="H40" s="1">
+        <f>H39+F40-F39</f>
+        <v>0.24305555555555552</v>
+      </c>
+      <c r="I40" s="1">
+        <f t="shared" ref="I40:K55" si="0">I39+G40-G39</f>
+        <v>6.3194444444444442E-2</v>
+      </c>
+      <c r="J40" s="1">
+        <f t="shared" si="0"/>
+        <v>0.3340277777777777</v>
+      </c>
+      <c r="K40" s="1">
+        <f t="shared" si="0"/>
+        <v>6.3194444444444442E-2</v>
+      </c>
+      <c r="L40" s="1">
+        <v>0.24513888888888888</v>
+      </c>
+      <c r="M40" s="1">
+        <v>9.2361111111111116E-2</v>
+      </c>
+      <c r="N40" s="1">
+        <f t="shared" ref="N40:N49" si="1">N41+L40-L41</f>
+        <v>0.25069444444444433</v>
+      </c>
+      <c r="O40" s="1">
+        <f t="shared" ref="O40:O49" si="2">O41+M40-M41</f>
+        <v>9.2361111111110908E-2</v>
+      </c>
+      <c r="P40" s="1">
+        <f t="shared" ref="P40:P49" si="3">P41+N40-N41</f>
+        <v>0.34166666666666656</v>
+      </c>
+      <c r="Q40" s="1">
+        <f t="shared" ref="Q40:Q49" si="4">Q41+O40-O41</f>
+        <v>9.2361111111111102E-2</v>
+      </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41">
@@ -2717,6 +2803,50 @@
       <c r="C41" t="s">
         <v>58</v>
       </c>
+      <c r="F41" s="1">
+        <v>0.2388888888888889</v>
+      </c>
+      <c r="G41" s="1">
+        <v>6.5277777777777782E-2</v>
+      </c>
+      <c r="H41" s="1">
+        <f t="shared" ref="H41:H61" si="5">H40+F41-F40</f>
+        <v>0.24444444444444441</v>
+      </c>
+      <c r="I41" s="1">
+        <f t="shared" si="0"/>
+        <v>6.388888888888887E-2</v>
+      </c>
+      <c r="J41" s="1">
+        <f t="shared" si="0"/>
+        <v>0.33541666666666653</v>
+      </c>
+      <c r="K41" s="1">
+        <f t="shared" si="0"/>
+        <v>6.3888888888888884E-2</v>
+      </c>
+      <c r="L41" s="1">
+        <v>0.24374999999999999</v>
+      </c>
+      <c r="M41" s="1">
+        <v>9.0972222222222218E-2</v>
+      </c>
+      <c r="N41" s="1">
+        <f t="shared" si="1"/>
+        <v>0.24930555555555547</v>
+      </c>
+      <c r="O41" s="1">
+        <f t="shared" si="2"/>
+        <v>9.0972222222222024E-2</v>
+      </c>
+      <c r="P41" s="1">
+        <f t="shared" si="3"/>
+        <v>0.34027777777777768</v>
+      </c>
+      <c r="Q41" s="1">
+        <f t="shared" si="4"/>
+        <v>9.0972222222222218E-2</v>
+      </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42">
@@ -2728,6 +2858,50 @@
       <c r="C42" t="s">
         <v>59</v>
       </c>
+      <c r="F42" s="1">
+        <v>0.24027777777777778</v>
+      </c>
+      <c r="G42" s="1">
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="H42" s="1">
+        <f t="shared" si="5"/>
+        <v>0.24583333333333326</v>
+      </c>
+      <c r="I42" s="1">
+        <f t="shared" si="0"/>
+        <v>6.5277777777777754E-2</v>
+      </c>
+      <c r="J42" s="1">
+        <f t="shared" si="0"/>
+        <v>0.33680555555555541</v>
+      </c>
+      <c r="K42" s="1">
+        <f t="shared" si="0"/>
+        <v>6.5277777777777782E-2</v>
+      </c>
+      <c r="L42" s="1">
+        <v>0.24236111111111111</v>
+      </c>
+      <c r="M42" s="1">
+        <v>8.9583333333333334E-2</v>
+      </c>
+      <c r="N42" s="1">
+        <f t="shared" si="1"/>
+        <v>0.24791666666666659</v>
+      </c>
+      <c r="O42" s="1">
+        <f t="shared" si="2"/>
+        <v>8.958333333333314E-2</v>
+      </c>
+      <c r="P42" s="1">
+        <f t="shared" si="3"/>
+        <v>0.3388888888888888</v>
+      </c>
+      <c r="Q42" s="1">
+        <f t="shared" si="4"/>
+        <v>8.958333333333332E-2</v>
+      </c>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43">
@@ -2739,6 +2913,50 @@
       <c r="C43" t="s">
         <v>60</v>
       </c>
+      <c r="F43" s="1">
+        <v>0.24166666666666667</v>
+      </c>
+      <c r="G43" s="1">
+        <v>6.805555555555555E-2</v>
+      </c>
+      <c r="H43" s="1">
+        <f t="shared" si="5"/>
+        <v>0.24722222222222215</v>
+      </c>
+      <c r="I43" s="1">
+        <f t="shared" si="0"/>
+        <v>6.6666666666666638E-2</v>
+      </c>
+      <c r="J43" s="1">
+        <f t="shared" si="0"/>
+        <v>0.33819444444444435</v>
+      </c>
+      <c r="K43" s="1">
+        <f t="shared" si="0"/>
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="L43" s="1">
+        <v>0.24166666666666667</v>
+      </c>
+      <c r="M43" s="1">
+        <v>8.8888888888888892E-2</v>
+      </c>
+      <c r="N43" s="1">
+        <f t="shared" si="1"/>
+        <v>0.24722222222222215</v>
+      </c>
+      <c r="O43" s="1">
+        <f t="shared" si="2"/>
+        <v>8.8888888888888712E-2</v>
+      </c>
+      <c r="P43" s="1">
+        <f t="shared" si="3"/>
+        <v>0.33819444444444435</v>
+      </c>
+      <c r="Q43" s="1">
+        <f t="shared" si="4"/>
+        <v>8.8888888888888878E-2</v>
+      </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A44">
@@ -2750,6 +2968,50 @@
       <c r="C44" t="s">
         <v>61</v>
       </c>
+      <c r="F44" s="1">
+        <v>0.24236111111111111</v>
+      </c>
+      <c r="G44" s="1">
+        <v>6.8750000000000006E-2</v>
+      </c>
+      <c r="H44" s="1">
+        <f t="shared" si="5"/>
+        <v>0.24791666666666659</v>
+      </c>
+      <c r="I44" s="1">
+        <f t="shared" si="0"/>
+        <v>6.736111111111108E-2</v>
+      </c>
+      <c r="J44" s="1">
+        <f t="shared" si="0"/>
+        <v>0.3388888888888888</v>
+      </c>
+      <c r="K44" s="1">
+        <f t="shared" si="0"/>
+        <v>6.7361111111111108E-2</v>
+      </c>
+      <c r="L44" s="1">
+        <v>0.24097222222222223</v>
+      </c>
+      <c r="M44" s="1">
+        <v>8.7499999999999994E-2</v>
+      </c>
+      <c r="N44" s="1">
+        <f t="shared" si="1"/>
+        <v>0.24652777777777771</v>
+      </c>
+      <c r="O44" s="1">
+        <f t="shared" si="2"/>
+        <v>8.7499999999999828E-2</v>
+      </c>
+      <c r="P44" s="1">
+        <f t="shared" si="3"/>
+        <v>0.33749999999999991</v>
+      </c>
+      <c r="Q44" s="1">
+        <f t="shared" si="4"/>
+        <v>8.7499999999999994E-2</v>
+      </c>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A45">
@@ -2761,6 +3023,50 @@
       <c r="C45" t="s">
         <v>62</v>
       </c>
+      <c r="F45" s="1">
+        <v>0.24305555555555555</v>
+      </c>
+      <c r="G45" s="1">
+        <v>6.9444444444444448E-2</v>
+      </c>
+      <c r="H45" s="1">
+        <f t="shared" si="5"/>
+        <v>0.24861111111111103</v>
+      </c>
+      <c r="I45" s="1">
+        <f t="shared" si="0"/>
+        <v>6.8055555555555508E-2</v>
+      </c>
+      <c r="J45" s="1">
+        <f t="shared" si="0"/>
+        <v>0.33958333333333324</v>
+      </c>
+      <c r="K45" s="1">
+        <f t="shared" si="0"/>
+        <v>6.805555555555555E-2</v>
+      </c>
+      <c r="L45" s="1">
+        <v>0.24027777777777778</v>
+      </c>
+      <c r="M45" s="1">
+        <v>8.6805555555555552E-2</v>
+      </c>
+      <c r="N45" s="1">
+        <f t="shared" si="1"/>
+        <v>0.24583333333333326</v>
+      </c>
+      <c r="O45" s="1">
+        <f t="shared" si="2"/>
+        <v>8.6805555555555386E-2</v>
+      </c>
+      <c r="P45" s="1">
+        <f t="shared" si="3"/>
+        <v>0.33680555555555547</v>
+      </c>
+      <c r="Q45" s="1">
+        <f t="shared" si="4"/>
+        <v>8.6805555555555552E-2</v>
+      </c>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A46">
@@ -2772,6 +3078,50 @@
       <c r="C46" t="s">
         <v>63</v>
       </c>
+      <c r="F46" s="1">
+        <v>0.24444444444444444</v>
+      </c>
+      <c r="G46" s="1">
+        <v>7.0833333333333331E-2</v>
+      </c>
+      <c r="H46" s="1">
+        <f t="shared" si="5"/>
+        <v>0.24999999999999992</v>
+      </c>
+      <c r="I46" s="1">
+        <f t="shared" si="0"/>
+        <v>6.9444444444444392E-2</v>
+      </c>
+      <c r="J46" s="1">
+        <f t="shared" si="0"/>
+        <v>0.34097222222222212</v>
+      </c>
+      <c r="K46" s="1">
+        <f t="shared" si="0"/>
+        <v>6.9444444444444448E-2</v>
+      </c>
+      <c r="L46" s="1">
+        <v>0.2388888888888889</v>
+      </c>
+      <c r="M46" s="1">
+        <v>8.611111111111111E-2</v>
+      </c>
+      <c r="N46" s="1">
+        <f t="shared" si="1"/>
+        <v>0.24444444444444435</v>
+      </c>
+      <c r="O46" s="1">
+        <f t="shared" si="2"/>
+        <v>8.6111111111110944E-2</v>
+      </c>
+      <c r="P46" s="1">
+        <f t="shared" si="3"/>
+        <v>0.33541666666666659</v>
+      </c>
+      <c r="Q46" s="1">
+        <f t="shared" si="4"/>
+        <v>8.611111111111111E-2</v>
+      </c>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A47">
@@ -2783,6 +3133,50 @@
       <c r="C47" t="s">
         <v>64</v>
       </c>
+      <c r="F47" s="1">
+        <v>0.24513888888888888</v>
+      </c>
+      <c r="G47" s="1">
+        <v>7.1527777777777773E-2</v>
+      </c>
+      <c r="H47" s="1">
+        <f t="shared" si="5"/>
+        <v>0.25069444444444433</v>
+      </c>
+      <c r="I47" s="1">
+        <f t="shared" si="0"/>
+        <v>7.0138888888888834E-2</v>
+      </c>
+      <c r="J47" s="1">
+        <f t="shared" si="0"/>
+        <v>0.34166666666666656</v>
+      </c>
+      <c r="K47" s="1">
+        <f t="shared" si="0"/>
+        <v>7.013888888888889E-2</v>
+      </c>
+      <c r="L47" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="M47" s="1">
+        <v>8.4722222222222227E-2</v>
+      </c>
+      <c r="N47" s="1">
+        <f t="shared" si="1"/>
+        <v>0.25555555555555542</v>
+      </c>
+      <c r="O47" s="1">
+        <f t="shared" si="2"/>
+        <v>8.472222222222206E-2</v>
+      </c>
+      <c r="P47" s="1">
+        <f t="shared" si="3"/>
+        <v>0.34652777777777766</v>
+      </c>
+      <c r="Q47" s="1">
+        <f t="shared" si="4"/>
+        <v>8.4722222222222213E-2</v>
+      </c>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A48">
@@ -2794,8 +3188,52 @@
       <c r="C48" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F48" s="1">
+        <v>0.24652777777777779</v>
+      </c>
+      <c r="G48" s="1">
+        <v>7.2222222222222215E-2</v>
+      </c>
+      <c r="H48" s="1">
+        <f t="shared" si="5"/>
+        <v>0.25208333333333321</v>
+      </c>
+      <c r="I48" s="1">
+        <f t="shared" si="0"/>
+        <v>7.0833333333333276E-2</v>
+      </c>
+      <c r="J48" s="1">
+        <f t="shared" si="0"/>
+        <v>0.34305555555555545</v>
+      </c>
+      <c r="K48" s="1">
+        <f t="shared" si="0"/>
+        <v>7.0833333333333331E-2</v>
+      </c>
+      <c r="L48" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="M48" s="1">
+        <v>8.4722222222222227E-2</v>
+      </c>
+      <c r="N48" s="1">
+        <f t="shared" si="1"/>
+        <v>0.25555555555555542</v>
+      </c>
+      <c r="O48" s="1">
+        <f t="shared" si="2"/>
+        <v>8.4722222222222074E-2</v>
+      </c>
+      <c r="P48" s="1">
+        <f t="shared" si="3"/>
+        <v>0.34652777777777766</v>
+      </c>
+      <c r="Q48" s="1">
+        <f t="shared" si="4"/>
+        <v>8.4722222222222213E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>2</v>
       </c>
@@ -2805,8 +3243,52 @@
       <c r="C49" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F49" s="1">
+        <v>0.24861111111111112</v>
+      </c>
+      <c r="G49" s="1">
+        <v>7.4305555555555555E-2</v>
+      </c>
+      <c r="H49" s="1">
+        <f t="shared" si="5"/>
+        <v>0.25416666666666654</v>
+      </c>
+      <c r="I49" s="1">
+        <f t="shared" si="0"/>
+        <v>7.2916666666666602E-2</v>
+      </c>
+      <c r="J49" s="1">
+        <f t="shared" si="0"/>
+        <v>0.34513888888888877</v>
+      </c>
+      <c r="K49" s="1">
+        <f t="shared" si="0"/>
+        <v>7.2916666666666657E-2</v>
+      </c>
+      <c r="L49" s="1">
+        <v>0.24722222222222223</v>
+      </c>
+      <c r="M49" s="1">
+        <v>8.2638888888888887E-2</v>
+      </c>
+      <c r="N49" s="1">
+        <f t="shared" si="1"/>
+        <v>0.25277777777777766</v>
+      </c>
+      <c r="O49" s="1">
+        <f t="shared" si="2"/>
+        <v>8.2638888888888748E-2</v>
+      </c>
+      <c r="P49" s="1">
+        <f t="shared" si="3"/>
+        <v>0.34374999999999989</v>
+      </c>
+      <c r="Q49" s="1">
+        <f t="shared" si="4"/>
+        <v>8.2638888888888887E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>2</v>
       </c>
@@ -2816,8 +3298,52 @@
       <c r="C50" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F50" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="G50" s="1">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="H50" s="1">
+        <f t="shared" si="5"/>
+        <v>0.25555555555555542</v>
+      </c>
+      <c r="I50" s="1">
+        <f t="shared" si="0"/>
+        <v>7.361111111111103E-2</v>
+      </c>
+      <c r="J50" s="1">
+        <f t="shared" si="0"/>
+        <v>0.34652777777777766</v>
+      </c>
+      <c r="K50" s="1">
+        <f t="shared" si="0"/>
+        <v>7.3611111111111099E-2</v>
+      </c>
+      <c r="L50" s="1">
+        <v>0.24652777777777779</v>
+      </c>
+      <c r="M50" s="1">
+        <v>8.1250000000000003E-2</v>
+      </c>
+      <c r="N50" s="1">
+        <f t="shared" ref="N50:N66" si="6">N51+L50-L51</f>
+        <v>0.25208333333333321</v>
+      </c>
+      <c r="O50" s="1">
+        <f t="shared" ref="O50:O66" si="7">O51+M50-M51</f>
+        <v>8.1249999999999864E-2</v>
+      </c>
+      <c r="P50" s="1">
+        <f t="shared" ref="P50:P66" si="8">P51+N50-N51</f>
+        <v>0.34305555555555545</v>
+      </c>
+      <c r="Q50" s="1">
+        <f t="shared" ref="Q50:Q66" si="9">Q51+O50-O51</f>
+        <v>8.1249999999999989E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>2</v>
       </c>
@@ -2827,8 +3353,52 @@
       <c r="C51" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F51" s="1">
+        <v>0.25069444444444444</v>
+      </c>
+      <c r="G51" s="1">
+        <v>7.5694444444444439E-2</v>
+      </c>
+      <c r="H51" s="1">
+        <f t="shared" si="5"/>
+        <v>0.25624999999999987</v>
+      </c>
+      <c r="I51" s="1">
+        <f t="shared" si="0"/>
+        <v>7.4305555555555472E-2</v>
+      </c>
+      <c r="J51" s="1">
+        <f t="shared" si="0"/>
+        <v>0.3472222222222221</v>
+      </c>
+      <c r="K51" s="1">
+        <f t="shared" si="0"/>
+        <v>7.4305555555555555E-2</v>
+      </c>
+      <c r="L51" s="1">
+        <v>0.24791666666666667</v>
+      </c>
+      <c r="M51" s="1">
+        <v>8.0555555555555561E-2</v>
+      </c>
+      <c r="N51" s="1">
+        <f t="shared" si="6"/>
+        <v>0.2534722222222221</v>
+      </c>
+      <c r="O51" s="1">
+        <f t="shared" si="7"/>
+        <v>8.0555555555555436E-2</v>
+      </c>
+      <c r="P51" s="1">
+        <f t="shared" si="8"/>
+        <v>0.34444444444444433</v>
+      </c>
+      <c r="Q51" s="1">
+        <f t="shared" si="9"/>
+        <v>8.0555555555555547E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>2</v>
       </c>
@@ -2838,8 +3408,55 @@
       <c r="C52" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" s="1">
+        <v>0.25208333333333333</v>
+      </c>
+      <c r="G52" s="1">
+        <v>7.6388888888888895E-2</v>
+      </c>
+      <c r="H52" s="1">
+        <f t="shared" si="5"/>
+        <v>0.25763888888888875</v>
+      </c>
+      <c r="I52" s="1">
+        <f t="shared" si="0"/>
+        <v>7.4999999999999914E-2</v>
+      </c>
+      <c r="J52" s="1">
+        <f t="shared" si="0"/>
+        <v>0.34861111111111098</v>
+      </c>
+      <c r="K52" s="1">
+        <f t="shared" si="0"/>
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="L52" s="1">
+        <v>0.24722222222222223</v>
+      </c>
+      <c r="M52" s="1">
+        <v>7.9861111111111105E-2</v>
+      </c>
+      <c r="N52" s="1">
+        <f t="shared" si="6"/>
+        <v>0.25277777777777766</v>
+      </c>
+      <c r="O52" s="1">
+        <f t="shared" si="7"/>
+        <v>7.9861111111110994E-2</v>
+      </c>
+      <c r="P52" s="1">
+        <f t="shared" si="8"/>
+        <v>0.34374999999999989</v>
+      </c>
+      <c r="Q52" s="1">
+        <f t="shared" si="9"/>
+        <v>7.9861111111111105E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>2</v>
       </c>
@@ -2849,8 +3466,55 @@
       <c r="C53" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="E53" t="s">
+        <v>14</v>
+      </c>
+      <c r="F53" s="1">
+        <v>0.25277777777777777</v>
+      </c>
+      <c r="G53" s="1">
+        <v>7.7083333333333337E-2</v>
+      </c>
+      <c r="H53" s="1">
+        <f t="shared" si="5"/>
+        <v>0.25833333333333319</v>
+      </c>
+      <c r="I53" s="1">
+        <f t="shared" si="0"/>
+        <v>7.5694444444444342E-2</v>
+      </c>
+      <c r="J53" s="1">
+        <f t="shared" si="0"/>
+        <v>0.34930555555555542</v>
+      </c>
+      <c r="K53" s="1">
+        <f t="shared" si="0"/>
+        <v>7.5694444444444439E-2</v>
+      </c>
+      <c r="L53" s="1">
+        <v>0.24652777777777779</v>
+      </c>
+      <c r="M53" s="1">
+        <v>7.9166666666666663E-2</v>
+      </c>
+      <c r="N53" s="1">
+        <f t="shared" si="6"/>
+        <v>0.25208333333333321</v>
+      </c>
+      <c r="O53" s="1">
+        <f t="shared" si="7"/>
+        <v>7.9166666666666552E-2</v>
+      </c>
+      <c r="P53" s="1">
+        <f t="shared" si="8"/>
+        <v>0.34305555555555545</v>
+      </c>
+      <c r="Q53" s="1">
+        <f t="shared" si="9"/>
+        <v>7.9166666666666663E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>2</v>
       </c>
@@ -2860,8 +3524,52 @@
       <c r="C54" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F54" s="1">
+        <v>0.25416666666666665</v>
+      </c>
+      <c r="G54" s="1">
+        <v>7.8472222222222221E-2</v>
+      </c>
+      <c r="H54" s="1">
+        <f t="shared" si="5"/>
+        <v>0.25972222222222208</v>
+      </c>
+      <c r="I54" s="1">
+        <f t="shared" si="0"/>
+        <v>7.7083333333333226E-2</v>
+      </c>
+      <c r="J54" s="1">
+        <f t="shared" si="0"/>
+        <v>0.35069444444444431</v>
+      </c>
+      <c r="K54" s="1">
+        <f t="shared" si="0"/>
+        <v>7.7083333333333337E-2</v>
+      </c>
+      <c r="L54" s="1">
+        <v>0.24513888888888888</v>
+      </c>
+      <c r="M54" s="1">
+        <v>7.7777777777777779E-2</v>
+      </c>
+      <c r="N54" s="1">
+        <f t="shared" si="6"/>
+        <v>0.25069444444444433</v>
+      </c>
+      <c r="O54" s="1">
+        <f t="shared" si="7"/>
+        <v>7.7777777777777668E-2</v>
+      </c>
+      <c r="P54" s="1">
+        <f t="shared" si="8"/>
+        <v>0.34166666666666656</v>
+      </c>
+      <c r="Q54" s="1">
+        <f t="shared" si="9"/>
+        <v>7.7777777777777765E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>2</v>
       </c>
@@ -2871,8 +3579,55 @@
       <c r="C55" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" s="1">
+        <v>0.25555555555555554</v>
+      </c>
+      <c r="G55" s="1">
+        <v>7.9166666666666663E-2</v>
+      </c>
+      <c r="H55" s="1">
+        <f t="shared" si="5"/>
+        <v>0.26111111111111096</v>
+      </c>
+      <c r="I55" s="1">
+        <f t="shared" si="0"/>
+        <v>7.7777777777777668E-2</v>
+      </c>
+      <c r="J55" s="1">
+        <f t="shared" si="0"/>
+        <v>0.35208333333333319</v>
+      </c>
+      <c r="K55" s="1">
+        <f t="shared" si="0"/>
+        <v>7.7777777777777779E-2</v>
+      </c>
+      <c r="L55" s="1">
+        <v>0.24444444444444444</v>
+      </c>
+      <c r="M55" s="1">
+        <v>7.7083333333333337E-2</v>
+      </c>
+      <c r="N55" s="1">
+        <f t="shared" si="6"/>
+        <v>0.24999999999999989</v>
+      </c>
+      <c r="O55" s="1">
+        <f t="shared" si="7"/>
+        <v>7.708333333333324E-2</v>
+      </c>
+      <c r="P55" s="1">
+        <f t="shared" si="8"/>
+        <v>0.34097222222222212</v>
+      </c>
+      <c r="Q55" s="1">
+        <f t="shared" si="9"/>
+        <v>7.7083333333333323E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>2</v>
       </c>
@@ -2882,8 +3637,52 @@
       <c r="C56" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F56" s="1">
+        <v>0.25624999999999998</v>
+      </c>
+      <c r="G56" s="1">
+        <v>7.9861111111111105E-2</v>
+      </c>
+      <c r="H56" s="1">
+        <f t="shared" si="5"/>
+        <v>0.2618055555555554</v>
+      </c>
+      <c r="I56" s="1">
+        <f t="shared" ref="I56:I61" si="10">I55+G56-G55</f>
+        <v>7.847222222222211E-2</v>
+      </c>
+      <c r="J56" s="1">
+        <f t="shared" ref="J56:J61" si="11">J55+H56-H55</f>
+        <v>0.35277777777777763</v>
+      </c>
+      <c r="K56" s="1">
+        <f t="shared" ref="K56:K61" si="12">K55+I56-I55</f>
+        <v>7.8472222222222221E-2</v>
+      </c>
+      <c r="L56" s="1">
+        <v>0.24652777777777779</v>
+      </c>
+      <c r="M56" s="1">
+        <v>7.5694444444444439E-2</v>
+      </c>
+      <c r="N56" s="1">
+        <f t="shared" si="6"/>
+        <v>0.25208333333333321</v>
+      </c>
+      <c r="O56" s="1">
+        <f t="shared" si="7"/>
+        <v>7.5694444444444356E-2</v>
+      </c>
+      <c r="P56" s="1">
+        <f t="shared" si="8"/>
+        <v>0.34305555555555545</v>
+      </c>
+      <c r="Q56" s="1">
+        <f t="shared" si="9"/>
+        <v>7.5694444444444439E-2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>2</v>
       </c>
@@ -2893,8 +3692,52 @@
       <c r="C57" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F57" s="1">
+        <v>0.25763888888888886</v>
+      </c>
+      <c r="G57" s="1">
+        <v>8.1250000000000003E-2</v>
+      </c>
+      <c r="H57" s="1">
+        <f t="shared" si="5"/>
+        <v>0.26319444444444429</v>
+      </c>
+      <c r="I57" s="1">
+        <f t="shared" si="10"/>
+        <v>7.9861111111110994E-2</v>
+      </c>
+      <c r="J57" s="1">
+        <f t="shared" si="11"/>
+        <v>0.35416666666666652</v>
+      </c>
+      <c r="K57" s="1">
+        <f t="shared" si="12"/>
+        <v>7.9861111111111105E-2</v>
+      </c>
+      <c r="L57" s="1">
+        <v>0.24583333333333332</v>
+      </c>
+      <c r="M57" s="1">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="N57" s="1">
+        <f t="shared" si="6"/>
+        <v>0.25138888888888877</v>
+      </c>
+      <c r="O57" s="1">
+        <f t="shared" si="7"/>
+        <v>7.4999999999999914E-2</v>
+      </c>
+      <c r="P57" s="1">
+        <f t="shared" si="8"/>
+        <v>0.34236111111111101</v>
+      </c>
+      <c r="Q57" s="1">
+        <f t="shared" si="9"/>
+        <v>7.4999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>2</v>
       </c>
@@ -2904,8 +3747,52 @@
       <c r="C58" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F58" s="1">
+        <v>0.2590277777777778</v>
+      </c>
+      <c r="G58" s="1">
+        <v>8.2638888888888887E-2</v>
+      </c>
+      <c r="H58" s="1">
+        <f t="shared" si="5"/>
+        <v>0.26458333333333328</v>
+      </c>
+      <c r="I58" s="1">
+        <f t="shared" si="10"/>
+        <v>8.1249999999999864E-2</v>
+      </c>
+      <c r="J58" s="1">
+        <f t="shared" si="11"/>
+        <v>0.35555555555555551</v>
+      </c>
+      <c r="K58" s="1">
+        <f t="shared" si="12"/>
+        <v>8.1249999999999989E-2</v>
+      </c>
+      <c r="L58" s="1">
+        <v>0.24513888888888888</v>
+      </c>
+      <c r="M58" s="1">
+        <v>7.4305555555555555E-2</v>
+      </c>
+      <c r="N58" s="1">
+        <f t="shared" si="6"/>
+        <v>0.25069444444444433</v>
+      </c>
+      <c r="O58" s="1">
+        <f t="shared" si="7"/>
+        <v>7.4305555555555472E-2</v>
+      </c>
+      <c r="P58" s="1">
+        <f t="shared" si="8"/>
+        <v>0.34166666666666656</v>
+      </c>
+      <c r="Q58" s="1">
+        <f t="shared" si="9"/>
+        <v>7.4305555555555541E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>2</v>
       </c>
@@ -2915,8 +3802,52 @@
       <c r="C59" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F59" s="1">
+        <v>0.26041666666666669</v>
+      </c>
+      <c r="G59" s="1">
+        <v>8.4027777777777785E-2</v>
+      </c>
+      <c r="H59" s="1">
+        <f t="shared" si="5"/>
+        <v>0.26597222222222211</v>
+      </c>
+      <c r="I59" s="1">
+        <f t="shared" si="10"/>
+        <v>8.2638888888888748E-2</v>
+      </c>
+      <c r="J59" s="1">
+        <f t="shared" si="11"/>
+        <v>0.3569444444444444</v>
+      </c>
+      <c r="K59" s="1">
+        <f t="shared" si="12"/>
+        <v>8.2638888888888887E-2</v>
+      </c>
+      <c r="L59" s="1">
+        <v>0.24444444444444444</v>
+      </c>
+      <c r="M59" s="1">
+        <v>7.3611111111111113E-2</v>
+      </c>
+      <c r="N59" s="1">
+        <f t="shared" si="6"/>
+        <v>0.24999999999999992</v>
+      </c>
+      <c r="O59" s="1">
+        <f t="shared" si="7"/>
+        <v>7.3611111111111044E-2</v>
+      </c>
+      <c r="P59" s="1">
+        <f t="shared" si="8"/>
+        <v>0.34097222222222212</v>
+      </c>
+      <c r="Q59" s="1">
+        <f t="shared" si="9"/>
+        <v>7.3611111111111099E-2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>2</v>
       </c>
@@ -2926,8 +3857,52 @@
       <c r="C60" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F60" s="1">
+        <v>0.26041666666666669</v>
+      </c>
+      <c r="G60" s="1">
+        <v>8.4027777777777785E-2</v>
+      </c>
+      <c r="H60" s="1">
+        <f t="shared" si="5"/>
+        <v>0.26597222222222211</v>
+      </c>
+      <c r="I60" s="1">
+        <f t="shared" si="10"/>
+        <v>8.2638888888888734E-2</v>
+      </c>
+      <c r="J60" s="1">
+        <f t="shared" si="11"/>
+        <v>0.35694444444444445</v>
+      </c>
+      <c r="K60" s="1">
+        <f t="shared" si="12"/>
+        <v>8.2638888888888887E-2</v>
+      </c>
+      <c r="L60" s="1">
+        <v>0.24374999999999999</v>
+      </c>
+      <c r="M60" s="1">
+        <v>7.2222222222222215E-2</v>
+      </c>
+      <c r="N60" s="1">
+        <f t="shared" si="6"/>
+        <v>0.24930555555555547</v>
+      </c>
+      <c r="O60" s="1">
+        <f t="shared" si="7"/>
+        <v>7.222222222222216E-2</v>
+      </c>
+      <c r="P60" s="1">
+        <f t="shared" si="8"/>
+        <v>0.34027777777777768</v>
+      </c>
+      <c r="Q60" s="1">
+        <f t="shared" si="9"/>
+        <v>7.2222222222222215E-2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>2</v>
       </c>
@@ -2937,8 +3912,52 @@
       <c r="C61" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F61" s="1">
+        <v>0.26111111111111113</v>
+      </c>
+      <c r="G61" s="1">
+        <v>8.4722222222222227E-2</v>
+      </c>
+      <c r="H61" s="1">
+        <f t="shared" si="5"/>
+        <v>0.26666666666666655</v>
+      </c>
+      <c r="I61" s="1">
+        <f t="shared" si="10"/>
+        <v>8.3333333333333176E-2</v>
+      </c>
+      <c r="J61" s="1">
+        <f t="shared" si="11"/>
+        <v>0.3576388888888889</v>
+      </c>
+      <c r="K61" s="1">
+        <f t="shared" si="12"/>
+        <v>8.3333333333333343E-2</v>
+      </c>
+      <c r="L61" s="1">
+        <v>0.24236111111111111</v>
+      </c>
+      <c r="M61" s="1">
+        <v>7.1527777777777773E-2</v>
+      </c>
+      <c r="N61" s="1">
+        <f t="shared" si="6"/>
+        <v>0.24791666666666659</v>
+      </c>
+      <c r="O61" s="1">
+        <f t="shared" si="7"/>
+        <v>7.1527777777777718E-2</v>
+      </c>
+      <c r="P61" s="1">
+        <f t="shared" si="8"/>
+        <v>0.3388888888888888</v>
+      </c>
+      <c r="Q61" s="1">
+        <f t="shared" si="9"/>
+        <v>7.1527777777777773E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>2</v>
       </c>
@@ -2948,8 +3967,51 @@
       <c r="C62" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" s="1">
+        <v>0.23819444444444443</v>
+      </c>
+      <c r="G62" s="1">
+        <v>8.5416666666666669E-2</v>
+      </c>
+      <c r="H62" s="1">
+        <v>0.24027777777777778</v>
+      </c>
+      <c r="I62" s="1">
+        <v>8.5416666666666669E-2</v>
+      </c>
+      <c r="J62" s="1">
+        <v>0.33750000000000002</v>
+      </c>
+      <c r="K62" s="1">
+        <v>8.5416666666666669E-2</v>
+      </c>
+      <c r="L62" s="1">
+        <v>0.24444444444444444</v>
+      </c>
+      <c r="M62" s="1">
+        <v>7.0833333333333331E-2</v>
+      </c>
+      <c r="N62" s="1">
+        <f t="shared" si="6"/>
+        <v>0.24999999999999992</v>
+      </c>
+      <c r="O62" s="1">
+        <f t="shared" si="7"/>
+        <v>7.0833333333333276E-2</v>
+      </c>
+      <c r="P62" s="1">
+        <f t="shared" si="8"/>
+        <v>0.34097222222222212</v>
+      </c>
+      <c r="Q62" s="1">
+        <f t="shared" si="9"/>
+        <v>7.0833333333333331E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>2</v>
       </c>
@@ -2959,8 +4021,52 @@
       <c r="C63" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F63" s="1">
+        <v>0.2388888888888889</v>
+      </c>
+      <c r="G63" s="1">
+        <v>8.611111111111111E-2</v>
+      </c>
+      <c r="H63" s="1">
+        <f>H62+F63-F62</f>
+        <v>0.24097222222222225</v>
+      </c>
+      <c r="I63" s="1">
+        <f t="shared" ref="I63:K63" si="13">I62+G63-G62</f>
+        <v>8.611111111111111E-2</v>
+      </c>
+      <c r="J63" s="1">
+        <f t="shared" si="13"/>
+        <v>0.33819444444444446</v>
+      </c>
+      <c r="K63" s="1">
+        <f>K62+I63-I62</f>
+        <v>8.611111111111111E-2</v>
+      </c>
+      <c r="L63" s="1">
+        <v>0.24374999999999999</v>
+      </c>
+      <c r="M63" s="1">
+        <v>7.013888888888889E-2</v>
+      </c>
+      <c r="N63" s="1">
+        <f t="shared" si="6"/>
+        <v>0.24930555555555547</v>
+      </c>
+      <c r="O63" s="1">
+        <f t="shared" si="7"/>
+        <v>7.0138888888888834E-2</v>
+      </c>
+      <c r="P63" s="1">
+        <f t="shared" si="8"/>
+        <v>0.34027777777777768</v>
+      </c>
+      <c r="Q63" s="1">
+        <f t="shared" si="9"/>
+        <v>7.013888888888889E-2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>2</v>
       </c>
@@ -2970,8 +4076,52 @@
       <c r="C64" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F64" s="1">
+        <v>0.24027777777777778</v>
+      </c>
+      <c r="G64" s="1">
+        <v>8.7499999999999994E-2</v>
+      </c>
+      <c r="H64" s="1">
+        <f>H63+F64-F63</f>
+        <v>0.24236111111111117</v>
+      </c>
+      <c r="I64" s="1">
+        <f t="shared" ref="I64:I67" si="14">I63+G64-G63</f>
+        <v>8.7499999999999994E-2</v>
+      </c>
+      <c r="J64" s="1">
+        <f t="shared" ref="J64:J67" si="15">J63+H64-H63</f>
+        <v>0.33958333333333335</v>
+      </c>
+      <c r="K64" s="1">
+        <f t="shared" ref="K64:K67" si="16">K63+I64-I63</f>
+        <v>8.7499999999999994E-2</v>
+      </c>
+      <c r="L64" s="1">
+        <v>0.24305555555555555</v>
+      </c>
+      <c r="M64" s="1">
+        <v>6.9444444444444448E-2</v>
+      </c>
+      <c r="N64" s="1">
+        <f t="shared" si="6"/>
+        <v>0.24861111111111103</v>
+      </c>
+      <c r="O64" s="1">
+        <f t="shared" si="7"/>
+        <v>6.9444444444444392E-2</v>
+      </c>
+      <c r="P64" s="1">
+        <f t="shared" si="8"/>
+        <v>0.33958333333333324</v>
+      </c>
+      <c r="Q64" s="1">
+        <f t="shared" si="9"/>
+        <v>6.9444444444444434E-2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>2</v>
       </c>
@@ -2981,8 +4131,52 @@
       <c r="C65" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F65" s="1">
+        <v>0.24166666666666667</v>
+      </c>
+      <c r="G65" s="1">
+        <v>8.819444444444445E-2</v>
+      </c>
+      <c r="H65" s="1">
+        <f>H64+F65-F64</f>
+        <v>0.24375000000000005</v>
+      </c>
+      <c r="I65" s="1">
+        <f t="shared" si="14"/>
+        <v>8.8194444444444436E-2</v>
+      </c>
+      <c r="J65" s="1">
+        <f t="shared" si="15"/>
+        <v>0.34097222222222223</v>
+      </c>
+      <c r="K65" s="1">
+        <f t="shared" si="16"/>
+        <v>8.8194444444444436E-2</v>
+      </c>
+      <c r="L65" s="1">
+        <v>0.24166666666666667</v>
+      </c>
+      <c r="M65" s="1">
+        <v>6.8750000000000006E-2</v>
+      </c>
+      <c r="N65" s="1">
+        <f t="shared" si="6"/>
+        <v>0.24722222222222215</v>
+      </c>
+      <c r="O65" s="1">
+        <f t="shared" si="7"/>
+        <v>6.8749999999999964E-2</v>
+      </c>
+      <c r="P65" s="1">
+        <f t="shared" si="8"/>
+        <v>0.3381944444444443</v>
+      </c>
+      <c r="Q65" s="1">
+        <f t="shared" si="9"/>
+        <v>6.8749999999999992E-2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>2</v>
       </c>
@@ -2992,8 +4186,52 @@
       <c r="C66" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F66" s="1">
+        <v>0.24305555555555555</v>
+      </c>
+      <c r="G66" s="1">
+        <v>8.9583333333333334E-2</v>
+      </c>
+      <c r="H66" s="1">
+        <f>H65+F66-F65</f>
+        <v>0.24513888888888893</v>
+      </c>
+      <c r="I66" s="1">
+        <f t="shared" si="14"/>
+        <v>8.9583333333333307E-2</v>
+      </c>
+      <c r="J66" s="1">
+        <f t="shared" si="15"/>
+        <v>0.34236111111111112</v>
+      </c>
+      <c r="K66" s="1">
+        <f t="shared" si="16"/>
+        <v>8.958333333333332E-2</v>
+      </c>
+      <c r="L66" s="1">
+        <v>0.24097222222222223</v>
+      </c>
+      <c r="M66" s="1">
+        <v>6.7361111111111108E-2</v>
+      </c>
+      <c r="N66" s="1">
+        <f t="shared" si="6"/>
+        <v>0.24652777777777773</v>
+      </c>
+      <c r="O66" s="1">
+        <f t="shared" si="7"/>
+        <v>6.736111111111108E-2</v>
+      </c>
+      <c r="P66" s="1">
+        <f t="shared" si="8"/>
+        <v>0.33749999999999986</v>
+      </c>
+      <c r="Q66" s="1">
+        <f t="shared" si="9"/>
+        <v>6.7361111111111094E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>2</v>
       </c>
@@ -3003,8 +4241,52 @@
       <c r="C67" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F67" s="1">
+        <v>0.24513888888888888</v>
+      </c>
+      <c r="G67" s="1">
+        <v>9.166666666666666E-2</v>
+      </c>
+      <c r="H67" s="1">
+        <f>H66+F67-F66</f>
+        <v>0.24722222222222226</v>
+      </c>
+      <c r="I67" s="1">
+        <f t="shared" si="14"/>
+        <v>9.1666666666666632E-2</v>
+      </c>
+      <c r="J67" s="1">
+        <f t="shared" si="15"/>
+        <v>0.34444444444444444</v>
+      </c>
+      <c r="K67" s="1">
+        <f t="shared" si="16"/>
+        <v>9.166666666666666E-2</v>
+      </c>
+      <c r="L67" s="1">
+        <v>0.23819444444444443</v>
+      </c>
+      <c r="M67" s="1">
+        <v>6.5277777777777782E-2</v>
+      </c>
+      <c r="N67" s="1">
+        <f>N68+L67-L68</f>
+        <v>0.24374999999999997</v>
+      </c>
+      <c r="O67" s="1">
+        <f t="shared" ref="O67:Q67" si="17">O68+M67-M68</f>
+        <v>6.5277777777777768E-2</v>
+      </c>
+      <c r="P67" s="1">
+        <f t="shared" si="17"/>
+        <v>0.33472222222222214</v>
+      </c>
+      <c r="Q67" s="1">
+        <f t="shared" si="17"/>
+        <v>6.5277777777777768E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>2</v>
       </c>
@@ -3013,6 +4295,42 @@
       </c>
       <c r="C68" t="s">
         <v>83</v>
+      </c>
+      <c r="F68" s="1">
+        <v>0.24791666666666667</v>
+      </c>
+      <c r="G68" s="1">
+        <v>9.4444444444444442E-2</v>
+      </c>
+      <c r="H68" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="I68" s="1">
+        <v>9.4444444444444442E-2</v>
+      </c>
+      <c r="J68" s="1">
+        <v>0.34722222222222221</v>
+      </c>
+      <c r="K68" s="1">
+        <v>9.4444444444444442E-2</v>
+      </c>
+      <c r="L68" s="1">
+        <v>0.2361111111111111</v>
+      </c>
+      <c r="M68" s="1">
+        <v>6.3194444444444442E-2</v>
+      </c>
+      <c r="N68" s="1">
+        <v>0.24166666666666667</v>
+      </c>
+      <c r="O68" s="1">
+        <v>6.3194444444444442E-2</v>
+      </c>
+      <c r="P68" s="1">
+        <v>0.33263888888888887</v>
+      </c>
+      <c r="Q68" s="1">
+        <v>6.3194444444444442E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>